<commit_message>
#8 Main Board Parts Search in Progress
</commit_message>
<xml_diff>
--- a/Design-Files/MotorDriver-v1.0/Deliverables/BOM/eSpark BOM.xlsx
+++ b/Design-Files/MotorDriver-v1.0/Deliverables/BOM/eSpark BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\hasanmehmood-motordriver\Design-Files\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\hasanmehmood-motordriver\Design-Files\MotorDriver-v1.0\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="349">
   <si>
     <t>Component list</t>
   </si>
@@ -1021,6 +1021,51 @@
   </si>
   <si>
     <t>High sensitivity wireless remote control receiving module RXB61 multiple frequency 315M.433MHZ</t>
+  </si>
+  <si>
+    <t>CL10B104KB8WPNC</t>
+  </si>
+  <si>
+    <t>GCM188R91H103KA37D</t>
+  </si>
+  <si>
+    <t>AC0603KRX7R8BB102</t>
+  </si>
+  <si>
+    <t>HMK212B7224KGHT</t>
+  </si>
+  <si>
+    <t>CRCW06031K00FKEA</t>
+  </si>
+  <si>
+    <t>CRCW06031K50FKEA</t>
+  </si>
+  <si>
+    <t>CRCW0603100KFKEA</t>
+  </si>
+  <si>
+    <t>CRCW060333K0JNEA</t>
+  </si>
+  <si>
+    <t>CRCW060315K0FKEA</t>
+  </si>
+  <si>
+    <t>CRCW06033K30FKEA</t>
+  </si>
+  <si>
+    <t>CRCW0603220RFKEA</t>
+  </si>
+  <si>
+    <t>RK73G1JTTD1002F</t>
+  </si>
+  <si>
+    <t>CRCW06038K20FKEA</t>
+  </si>
+  <si>
+    <t>CRCW0603150RFKEA</t>
+  </si>
+  <si>
+    <t>CRCW0603100RFKEB</t>
   </si>
 </sst>
 </file>
@@ -1032,7 +1077,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1041,24 +1086,31 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color indexed="13"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="24"/>
       <color indexed="10"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="24"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1066,7 +1118,7 @@
       <sz val="12"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1074,21 +1126,21 @@
       <sz val="12"/>
       <color theme="0"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color indexed="10"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1096,65 +1148,65 @@
       <sz val="10"/>
       <color theme="0"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="0"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color indexed="10"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="0"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color indexed="10"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1162,7 +1214,7 @@
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1171,13 +1223,13 @@
       <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1185,13 +1237,14 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1199,13 +1252,13 @@
       <sz val="12"/>
       <color indexed="13"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1470,94 +1523,91 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1566,25 +1616,28 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1592,72 +1645,72 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="18" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
@@ -1667,18 +1720,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2012,7 +2067,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S65"/>
+  <dimension ref="A1:V65"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="1" customWidth="1"/>
@@ -2033,9 +2088,10 @@
     <col min="17" max="17" width="20.140625" customWidth="1"/>
     <col min="18" max="18" width="16.5703125" customWidth="1"/>
     <col min="19" max="19" width="26.85546875" customWidth="1"/>
+    <col min="21" max="21" width="21.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:22">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2056,7 +2112,7 @@
       <c r="R1" s="64"/>
       <c r="S1" s="65"/>
     </row>
-    <row r="2" spans="1:19" ht="31.5">
+    <row r="2" spans="1:22" ht="31.5">
       <c r="A2" s="2"/>
       <c r="B2" s="5"/>
       <c r="C2" s="6"/>
@@ -2081,7 +2137,7 @@
       <c r="R2" s="9"/>
       <c r="S2" s="56"/>
     </row>
-    <row r="3" spans="1:19">
+    <row r="3" spans="1:22">
       <c r="A3" s="2"/>
       <c r="B3" s="10"/>
       <c r="C3" s="11"/>
@@ -2106,7 +2162,7 @@
       <c r="R3" s="13"/>
       <c r="S3" s="68"/>
     </row>
-    <row r="4" spans="1:19">
+    <row r="4" spans="1:22">
       <c r="A4" s="2"/>
       <c r="B4" s="10"/>
       <c r="C4" s="11"/>
@@ -2131,7 +2187,7 @@
       <c r="R4" s="17"/>
       <c r="S4" s="69"/>
     </row>
-    <row r="5" spans="1:19">
+    <row r="5" spans="1:22">
       <c r="A5" s="2"/>
       <c r="B5" s="10"/>
       <c r="C5" s="11"/>
@@ -2156,7 +2212,7 @@
       <c r="R5" s="17"/>
       <c r="S5" s="69"/>
     </row>
-    <row r="6" spans="1:19">
+    <row r="6" spans="1:22">
       <c r="A6" s="2"/>
       <c r="B6" s="18"/>
       <c r="C6" s="19"/>
@@ -2177,7 +2233,7 @@
       <c r="R6" s="17"/>
       <c r="S6" s="69"/>
     </row>
-    <row r="7" spans="1:19">
+    <row r="7" spans="1:22">
       <c r="A7" s="2"/>
       <c r="B7" s="22"/>
       <c r="C7" s="23"/>
@@ -2198,7 +2254,7 @@
       <c r="R7" s="26"/>
       <c r="S7" s="69"/>
     </row>
-    <row r="8" spans="1:19">
+    <row r="8" spans="1:22">
       <c r="A8" s="2"/>
       <c r="B8" s="27"/>
       <c r="C8" s="28"/>
@@ -2219,7 +2275,7 @@
       <c r="R8" s="26"/>
       <c r="S8" s="69"/>
     </row>
-    <row r="9" spans="1:19">
+    <row r="9" spans="1:22">
       <c r="A9" s="2"/>
       <c r="B9" s="31" t="s">
         <v>7</v>
@@ -2276,7 +2332,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="24">
+    <row r="10" spans="1:22" ht="24">
       <c r="A10" s="2"/>
       <c r="B10" s="32">
         <f t="shared" ref="B10:B17" si="0">ROW(B10)-ROW($B$9)</f>
@@ -2332,7 +2388,7 @@
       <c r="R10" s="34"/>
       <c r="S10" s="57"/>
     </row>
-    <row r="11" spans="1:19">
+    <row r="11" spans="1:22">
       <c r="A11" s="2"/>
       <c r="B11" s="35">
         <f t="shared" si="0"/>
@@ -2387,8 +2443,14 @@
       </c>
       <c r="R11" s="37"/>
       <c r="S11" s="37"/>
-    </row>
-    <row r="12" spans="1:19" ht="36">
+      <c r="U11" s="74" t="s">
+        <v>334</v>
+      </c>
+      <c r="V11" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" ht="36">
       <c r="A12" s="2"/>
       <c r="B12" s="32">
         <f t="shared" si="0"/>
@@ -2443,8 +2505,11 @@
       </c>
       <c r="R12" s="34"/>
       <c r="S12" s="57"/>
-    </row>
-    <row r="13" spans="1:19">
+      <c r="V12" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22">
       <c r="A13" s="2"/>
       <c r="B13" s="35">
         <f t="shared" si="0"/>
@@ -2499,8 +2564,14 @@
       </c>
       <c r="R13" s="37"/>
       <c r="S13" s="37"/>
-    </row>
-    <row r="14" spans="1:19" ht="24">
+      <c r="U13" s="74" t="s">
+        <v>335</v>
+      </c>
+      <c r="V13" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" ht="24">
       <c r="A14" s="2"/>
       <c r="B14" s="32">
         <f t="shared" si="0"/>
@@ -2555,8 +2626,14 @@
       </c>
       <c r="R14" s="34"/>
       <c r="S14" s="57"/>
-    </row>
-    <row r="15" spans="1:19" ht="36">
+      <c r="U14" s="74" t="s">
+        <v>336</v>
+      </c>
+      <c r="V14" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" ht="36">
       <c r="A15" s="2"/>
       <c r="B15" s="35">
         <f t="shared" si="0"/>
@@ -2611,8 +2688,11 @@
       </c>
       <c r="R15" s="37"/>
       <c r="S15" s="37"/>
-    </row>
-    <row r="16" spans="1:19">
+      <c r="V15" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22">
       <c r="A16" s="2"/>
       <c r="B16" s="32">
         <f t="shared" si="0"/>
@@ -2667,8 +2747,14 @@
       </c>
       <c r="R16" s="34"/>
       <c r="S16" s="57"/>
-    </row>
-    <row r="17" spans="1:19" ht="24">
+      <c r="U16" s="74" t="s">
+        <v>337</v>
+      </c>
+      <c r="V16" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" ht="24">
       <c r="A17" s="2"/>
       <c r="B17" s="35">
         <f t="shared" si="0"/>
@@ -2723,8 +2809,11 @@
       </c>
       <c r="R17" s="37"/>
       <c r="S17" s="37"/>
-    </row>
-    <row r="18" spans="1:19" ht="24">
+      <c r="V17" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" ht="24">
       <c r="A18" s="2"/>
       <c r="B18" s="35">
         <f t="shared" ref="B18:B63" si="3">ROW(B18)-ROW($B$9)</f>
@@ -2779,8 +2868,11 @@
       </c>
       <c r="R18" s="37"/>
       <c r="S18" s="37"/>
-    </row>
-    <row r="19" spans="1:19">
+      <c r="V18" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22">
       <c r="A19" s="2"/>
       <c r="B19" s="32">
         <f t="shared" si="3"/>
@@ -2835,8 +2927,11 @@
       </c>
       <c r="R19" s="34"/>
       <c r="S19" s="57"/>
-    </row>
-    <row r="20" spans="1:19" ht="36">
+      <c r="V19" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" ht="36">
       <c r="A20" s="2"/>
       <c r="B20" s="35">
         <f t="shared" si="3"/>
@@ -2891,8 +2986,11 @@
       </c>
       <c r="R20" s="37"/>
       <c r="S20" s="37"/>
-    </row>
-    <row r="21" spans="1:19" ht="60">
+      <c r="V20" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" ht="60">
       <c r="A21" s="2"/>
       <c r="B21" s="32">
         <f t="shared" si="3"/>
@@ -2945,8 +3043,11 @@
       </c>
       <c r="R21" s="34"/>
       <c r="S21" s="57"/>
-    </row>
-    <row r="22" spans="1:19" ht="60">
+      <c r="V21" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" ht="60">
       <c r="A22" s="2"/>
       <c r="B22" s="35">
         <f t="shared" si="3"/>
@@ -2999,8 +3100,11 @@
       </c>
       <c r="R22" s="37"/>
       <c r="S22" s="37"/>
-    </row>
-    <row r="23" spans="1:19" ht="24">
+      <c r="V22" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" ht="24">
       <c r="A23" s="2"/>
       <c r="B23" s="32">
         <f t="shared" si="3"/>
@@ -3053,8 +3157,11 @@
       </c>
       <c r="R23" s="34"/>
       <c r="S23" s="57"/>
-    </row>
-    <row r="24" spans="1:19" ht="48">
+      <c r="V23" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" ht="48">
       <c r="A24" s="2"/>
       <c r="B24" s="35">
         <f t="shared" si="3"/>
@@ -3107,8 +3214,11 @@
       </c>
       <c r="R24" s="37"/>
       <c r="S24" s="37"/>
-    </row>
-    <row r="25" spans="1:19">
+      <c r="V24" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22">
       <c r="A25" s="2"/>
       <c r="B25" s="32">
         <f t="shared" si="3"/>
@@ -3161,8 +3271,11 @@
       </c>
       <c r="R25" s="34"/>
       <c r="S25" s="57"/>
-    </row>
-    <row r="26" spans="1:19" ht="24">
+      <c r="V25" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" ht="24">
       <c r="A26" s="2"/>
       <c r="B26" s="35">
         <f t="shared" si="3"/>
@@ -3215,8 +3328,11 @@
       </c>
       <c r="R26" s="37"/>
       <c r="S26" s="37"/>
-    </row>
-    <row r="27" spans="1:19" ht="48">
+      <c r="V26" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" ht="48">
       <c r="A27" s="2"/>
       <c r="B27" s="32">
         <f t="shared" si="3"/>
@@ -3272,8 +3388,11 @@
         <v>130</v>
       </c>
       <c r="S27" s="58"/>
-    </row>
-    <row r="28" spans="1:19" ht="24">
+      <c r="V27" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" ht="24">
       <c r="A28" s="2"/>
       <c r="B28" s="35">
         <f t="shared" si="3"/>
@@ -3328,8 +3447,11 @@
       </c>
       <c r="R28" s="37"/>
       <c r="S28" s="37"/>
-    </row>
-    <row r="29" spans="1:19" ht="36">
+      <c r="V28" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" ht="36">
       <c r="A29" s="2"/>
       <c r="B29" s="32">
         <f t="shared" si="3"/>
@@ -3385,8 +3507,11 @@
         <v>130</v>
       </c>
       <c r="S29" s="58"/>
-    </row>
-    <row r="30" spans="1:19" ht="48">
+      <c r="V29" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" ht="48">
       <c r="A30" s="2"/>
       <c r="B30" s="35">
         <f t="shared" si="3"/>
@@ -3441,8 +3566,11 @@
       </c>
       <c r="R30" s="37"/>
       <c r="S30" s="37"/>
-    </row>
-    <row r="31" spans="1:19" ht="36">
+      <c r="V30" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" ht="36">
       <c r="A31" s="2"/>
       <c r="B31" s="32">
         <f t="shared" si="3"/>
@@ -3497,8 +3625,11 @@
       </c>
       <c r="R31" s="34"/>
       <c r="S31" s="57"/>
-    </row>
-    <row r="32" spans="1:19">
+      <c r="V31" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22">
       <c r="A32" s="2"/>
       <c r="B32" s="35">
         <f t="shared" si="3"/>
@@ -3553,8 +3684,11 @@
       </c>
       <c r="R32" s="37"/>
       <c r="S32" s="37"/>
-    </row>
-    <row r="33" spans="1:19" ht="24">
+      <c r="V32" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" ht="24">
       <c r="A33" s="2"/>
       <c r="B33" s="32">
         <f t="shared" si="3"/>
@@ -3609,8 +3743,11 @@
       </c>
       <c r="R33" s="34"/>
       <c r="S33" s="57"/>
-    </row>
-    <row r="34" spans="1:19" ht="24">
+      <c r="V33" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" ht="24">
       <c r="A34" s="2"/>
       <c r="B34" s="35">
         <f t="shared" si="3"/>
@@ -3665,8 +3802,11 @@
       </c>
       <c r="R34" s="37"/>
       <c r="S34" s="37"/>
-    </row>
-    <row r="35" spans="1:19" ht="36">
+      <c r="V34" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" ht="36">
       <c r="A35" s="2"/>
       <c r="B35" s="32">
         <f t="shared" si="3"/>
@@ -3721,8 +3861,11 @@
       </c>
       <c r="R35" s="34"/>
       <c r="S35" s="57"/>
-    </row>
-    <row r="36" spans="1:19" ht="36">
+      <c r="V35" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" ht="36">
       <c r="A36" s="2"/>
       <c r="B36" s="35">
         <f t="shared" si="3"/>
@@ -3777,8 +3920,11 @@
       </c>
       <c r="R36" s="37"/>
       <c r="S36" s="37"/>
-    </row>
-    <row r="37" spans="1:19" ht="25.5">
+      <c r="V36" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" ht="25.5">
       <c r="A37" s="2"/>
       <c r="B37" s="32">
         <f t="shared" si="3"/>
@@ -3833,8 +3979,11 @@
       </c>
       <c r="R37" s="34"/>
       <c r="S37" s="57"/>
-    </row>
-    <row r="38" spans="1:19">
+      <c r="V37" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22">
       <c r="A38" s="2"/>
       <c r="B38" s="35">
         <f t="shared" si="3"/>
@@ -3889,8 +4038,14 @@
       </c>
       <c r="R38" s="37"/>
       <c r="S38" s="37"/>
-    </row>
-    <row r="39" spans="1:19">
+      <c r="U38" s="74" t="s">
+        <v>338</v>
+      </c>
+      <c r="V38" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22">
       <c r="A39" s="2"/>
       <c r="B39" s="32">
         <f t="shared" si="3"/>
@@ -3945,8 +4100,14 @@
       </c>
       <c r="R39" s="34"/>
       <c r="S39" s="57"/>
-    </row>
-    <row r="40" spans="1:19">
+      <c r="U39" s="74" t="s">
+        <v>339</v>
+      </c>
+      <c r="V39" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22">
       <c r="A40" s="2"/>
       <c r="B40" s="35">
         <f t="shared" si="3"/>
@@ -4001,8 +4162,14 @@
       </c>
       <c r="R40" s="37"/>
       <c r="S40" s="37"/>
-    </row>
-    <row r="41" spans="1:19">
+      <c r="U40" s="74" t="s">
+        <v>340</v>
+      </c>
+      <c r="V40" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22">
       <c r="A41" s="2"/>
       <c r="B41" s="32">
         <f t="shared" si="3"/>
@@ -4057,8 +4224,14 @@
       </c>
       <c r="R41" s="34"/>
       <c r="S41" s="57"/>
-    </row>
-    <row r="42" spans="1:19">
+      <c r="U41" s="74" t="s">
+        <v>341</v>
+      </c>
+      <c r="V41" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22">
       <c r="A42" s="2"/>
       <c r="B42" s="35">
         <f t="shared" si="3"/>
@@ -4113,8 +4286,14 @@
       </c>
       <c r="R42" s="37"/>
       <c r="S42" s="37"/>
-    </row>
-    <row r="43" spans="1:19">
+      <c r="U42" s="74" t="s">
+        <v>342</v>
+      </c>
+      <c r="V42" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22">
       <c r="A43" s="2"/>
       <c r="B43" s="32">
         <f t="shared" si="3"/>
@@ -4169,8 +4348,14 @@
       </c>
       <c r="R43" s="34"/>
       <c r="S43" s="57"/>
-    </row>
-    <row r="44" spans="1:19">
+      <c r="U43" s="74" t="s">
+        <v>343</v>
+      </c>
+      <c r="V43" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="44" spans="1:22">
       <c r="A44" s="2"/>
       <c r="B44" s="35">
         <f t="shared" si="3"/>
@@ -4225,8 +4410,14 @@
       </c>
       <c r="R44" s="37"/>
       <c r="S44" s="37"/>
-    </row>
-    <row r="45" spans="1:19">
+      <c r="U44" s="74" t="s">
+        <v>344</v>
+      </c>
+      <c r="V44" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22">
       <c r="A45" s="2"/>
       <c r="B45" s="32">
         <f t="shared" si="3"/>
@@ -4281,8 +4472,14 @@
       </c>
       <c r="R45" s="34"/>
       <c r="S45" s="57"/>
-    </row>
-    <row r="46" spans="1:19">
+      <c r="U45" s="74" t="s">
+        <v>345</v>
+      </c>
+      <c r="V45" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22">
       <c r="A46" s="2"/>
       <c r="B46" s="35">
         <f t="shared" si="3"/>
@@ -4337,8 +4534,14 @@
       </c>
       <c r="R46" s="37"/>
       <c r="S46" s="37"/>
-    </row>
-    <row r="47" spans="1:19">
+      <c r="U46" s="74" t="s">
+        <v>346</v>
+      </c>
+      <c r="V46" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22">
       <c r="A47" s="2"/>
       <c r="B47" s="32">
         <f t="shared" si="3"/>
@@ -4393,8 +4596,14 @@
       </c>
       <c r="R47" s="34"/>
       <c r="S47" s="57"/>
-    </row>
-    <row r="48" spans="1:19">
+      <c r="U47" s="74" t="s">
+        <v>347</v>
+      </c>
+      <c r="V47" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22">
       <c r="A48" s="2"/>
       <c r="B48" s="35">
         <f t="shared" si="3"/>
@@ -4449,8 +4658,14 @@
       </c>
       <c r="R48" s="37"/>
       <c r="S48" s="37"/>
-    </row>
-    <row r="49" spans="1:19" ht="24">
+      <c r="U48" s="74" t="s">
+        <v>348</v>
+      </c>
+      <c r="V48" s="75" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="49" spans="1:22" ht="24">
       <c r="A49" s="2"/>
       <c r="B49" s="32">
         <f t="shared" si="3"/>
@@ -4505,8 +4720,11 @@
       </c>
       <c r="R49" s="34"/>
       <c r="S49" s="57"/>
-    </row>
-    <row r="50" spans="1:19" ht="24">
+      <c r="V49" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="50" spans="1:22" ht="24">
       <c r="A50" s="2"/>
       <c r="B50" s="35">
         <f t="shared" si="3"/>
@@ -4561,8 +4779,11 @@
       </c>
       <c r="R50" s="37"/>
       <c r="S50" s="37"/>
-    </row>
-    <row r="51" spans="1:19" ht="24">
+      <c r="V50" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="51" spans="1:22" ht="24">
       <c r="A51" s="2"/>
       <c r="B51" s="32">
         <f t="shared" si="3"/>
@@ -4617,8 +4838,11 @@
       </c>
       <c r="R51" s="34"/>
       <c r="S51" s="57"/>
-    </row>
-    <row r="52" spans="1:19" ht="36">
+      <c r="V51" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="52" spans="1:22" ht="36">
       <c r="A52" s="2"/>
       <c r="B52" s="35">
         <f t="shared" si="3"/>
@@ -4673,8 +4897,11 @@
       </c>
       <c r="R52" s="37"/>
       <c r="S52" s="37"/>
-    </row>
-    <row r="53" spans="1:19" ht="36">
+      <c r="V52" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="53" spans="1:22" ht="36">
       <c r="A53" s="2"/>
       <c r="B53" s="32">
         <f t="shared" si="3"/>
@@ -4729,8 +4956,11 @@
       </c>
       <c r="R53" s="34"/>
       <c r="S53" s="57"/>
-    </row>
-    <row r="54" spans="1:19">
+      <c r="V53" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="54" spans="1:22">
       <c r="A54" s="2"/>
       <c r="B54" s="35">
         <f t="shared" si="3"/>
@@ -4785,8 +5015,11 @@
       </c>
       <c r="R54" s="37"/>
       <c r="S54" s="37"/>
-    </row>
-    <row r="55" spans="1:19">
+      <c r="V54" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="55" spans="1:22">
       <c r="A55" s="2"/>
       <c r="B55" s="32">
         <f t="shared" si="3"/>
@@ -4841,8 +5074,11 @@
       </c>
       <c r="R55" s="34"/>
       <c r="S55" s="57"/>
-    </row>
-    <row r="56" spans="1:19" ht="24">
+      <c r="V55" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="56" spans="1:22" ht="24">
       <c r="A56" s="2"/>
       <c r="B56" s="35">
         <f t="shared" si="3"/>
@@ -4897,8 +5133,11 @@
       </c>
       <c r="R56" s="37"/>
       <c r="S56" s="37"/>
-    </row>
-    <row r="57" spans="1:19">
+      <c r="V56" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="57" spans="1:22">
       <c r="A57" s="2"/>
       <c r="B57" s="32">
         <f t="shared" si="3"/>
@@ -4953,8 +5192,11 @@
       </c>
       <c r="R57" s="34"/>
       <c r="S57" s="57"/>
-    </row>
-    <row r="58" spans="1:19" ht="24">
+      <c r="V57" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="58" spans="1:22" ht="24">
       <c r="A58" s="2"/>
       <c r="B58" s="35">
         <f t="shared" si="3"/>
@@ -5009,8 +5251,11 @@
       </c>
       <c r="R58" s="37"/>
       <c r="S58" s="37"/>
-    </row>
-    <row r="59" spans="1:19">
+      <c r="V58" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="59" spans="1:22">
       <c r="A59" s="2"/>
       <c r="B59" s="32">
         <f t="shared" si="3"/>
@@ -5065,8 +5310,11 @@
       </c>
       <c r="R59" s="34"/>
       <c r="S59" s="57"/>
-    </row>
-    <row r="60" spans="1:19" ht="36">
+      <c r="V59" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="60" spans="1:22" ht="36">
       <c r="A60" s="2"/>
       <c r="B60" s="32">
         <f t="shared" si="3"/>
@@ -5121,8 +5369,11 @@
       </c>
       <c r="R60" s="34"/>
       <c r="S60" s="57"/>
-    </row>
-    <row r="61" spans="1:19" ht="36">
+      <c r="V60" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="61" spans="1:22" ht="36">
       <c r="A61" s="2"/>
       <c r="B61" s="32">
         <f t="shared" si="3"/>
@@ -5177,8 +5428,11 @@
       </c>
       <c r="R61" s="34"/>
       <c r="S61" s="57"/>
-    </row>
-    <row r="62" spans="1:19" ht="24">
+      <c r="V61" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="62" spans="1:22" ht="24">
       <c r="A62" s="2"/>
       <c r="B62" s="32">
         <f t="shared" si="3"/>
@@ -5233,8 +5487,11 @@
       </c>
       <c r="R62" s="34"/>
       <c r="S62" s="57"/>
-    </row>
-    <row r="63" spans="1:19" ht="36">
+      <c r="V62" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="63" spans="1:22" ht="36">
       <c r="A63" s="2"/>
       <c r="B63" s="32">
         <f t="shared" si="3"/>
@@ -5289,8 +5546,11 @@
       </c>
       <c r="R63" s="34"/>
       <c r="S63" s="57"/>
-    </row>
-    <row r="64" spans="1:19" ht="18.75">
+      <c r="V63" s="74" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="64" spans="1:22" ht="18.75">
       <c r="A64" s="2"/>
       <c r="B64" s="41"/>
       <c r="C64" s="42"/>
@@ -5403,9 +5663,24 @@
     <hyperlink ref="O61" r:id="rId50"/>
     <hyperlink ref="O62" r:id="rId51"/>
     <hyperlink ref="O63" r:id="rId52"/>
+    <hyperlink ref="V11" r:id="rId53"/>
+    <hyperlink ref="V13" r:id="rId54"/>
+    <hyperlink ref="V14" r:id="rId55"/>
+    <hyperlink ref="V16" r:id="rId56"/>
+    <hyperlink ref="V38" r:id="rId57"/>
+    <hyperlink ref="V39" r:id="rId58"/>
+    <hyperlink ref="V40" r:id="rId59"/>
+    <hyperlink ref="V41" r:id="rId60"/>
+    <hyperlink ref="V42" r:id="rId61"/>
+    <hyperlink ref="V43" r:id="rId62"/>
+    <hyperlink ref="V44" r:id="rId63"/>
+    <hyperlink ref="V45" r:id="rId64"/>
+    <hyperlink ref="V46" r:id="rId65"/>
+    <hyperlink ref="V47" r:id="rId66"/>
+    <hyperlink ref="V48" r:id="rId67"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <drawing r:id="rId53"/>
+  <drawing r:id="rId68"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#8 Parts added in Library
</commit_message>
<xml_diff>
--- a/Design-Files/MotorDriver-v1.0/Deliverables/BOM/eSpark BOM.xlsx
+++ b/Design-Files/MotorDriver-v1.0/Deliverables/BOM/eSpark BOM.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="375">
   <si>
     <t>Component list</t>
   </si>
@@ -1015,12 +1015,6 @@
   </si>
   <si>
     <t>63A Glass Tube Fuse 6.3A 250V - Fuses</t>
-  </si>
-  <si>
-    <t>RF Module</t>
-  </si>
-  <si>
-    <t>High sensitivity wireless remote control receiving module RXB61 multiple frequency 315M.433MHZ</t>
   </si>
   <si>
     <t>CL10B104KB8WPNC</t>
@@ -1145,6 +1139,18 @@
   </si>
   <si>
     <t>CSL0902BT1C</t>
+  </si>
+  <si>
+    <t>Footprint Change</t>
+  </si>
+  <si>
+    <t>Pins not confirm</t>
+  </si>
+  <si>
+    <t>PTC10LV10-104A2020</t>
+  </si>
+  <si>
+    <t>Already industrial</t>
   </si>
 </sst>
 </file>
@@ -1156,12 +1162,19 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1349,6 +1362,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -1617,94 +1637,91 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1713,25 +1730,28 @@
     <xf numFmtId="0" fontId="20" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1739,74 +1759,82 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="20" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
@@ -1816,30 +1844,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2173,7 +2201,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:W65"/>
+  <dimension ref="A1:X64"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="1" customWidth="1"/>
@@ -2196,9 +2224,10 @@
     <col min="19" max="19" width="26.85546875" customWidth="1"/>
     <col min="21" max="21" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23">
+    <row r="1" spans="1:24">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2209,17 +2238,17 @@
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66"/>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="67"/>
-    </row>
-    <row r="2" spans="1:23" ht="31.5">
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="70"/>
+      <c r="O1" s="70"/>
+      <c r="P1" s="70"/>
+      <c r="Q1" s="70"/>
+      <c r="R1" s="70"/>
+      <c r="S1" s="71"/>
+    </row>
+    <row r="2" spans="1:24" ht="31.5">
       <c r="A2" s="2"/>
       <c r="B2" s="5"/>
       <c r="C2" s="6"/>
@@ -2244,7 +2273,7 @@
       <c r="R2" s="9"/>
       <c r="S2" s="56"/>
     </row>
-    <row r="3" spans="1:23">
+    <row r="3" spans="1:24">
       <c r="A3" s="2"/>
       <c r="B3" s="10"/>
       <c r="C3" s="11"/>
@@ -2267,9 +2296,9 @@
       <c r="P3" s="13"/>
       <c r="Q3" s="13"/>
       <c r="R3" s="13"/>
-      <c r="S3" s="70"/>
-    </row>
-    <row r="4" spans="1:23">
+      <c r="S3" s="74"/>
+    </row>
+    <row r="4" spans="1:24">
       <c r="A4" s="2"/>
       <c r="B4" s="10"/>
       <c r="C4" s="11"/>
@@ -2292,9 +2321,9 @@
       <c r="P4" s="17"/>
       <c r="Q4" s="17"/>
       <c r="R4" s="17"/>
-      <c r="S4" s="71"/>
-    </row>
-    <row r="5" spans="1:23">
+      <c r="S4" s="75"/>
+    </row>
+    <row r="5" spans="1:24">
       <c r="A5" s="2"/>
       <c r="B5" s="10"/>
       <c r="C5" s="11"/>
@@ -2317,9 +2346,9 @@
       <c r="P5" s="17"/>
       <c r="Q5" s="17"/>
       <c r="R5" s="17"/>
-      <c r="S5" s="71"/>
-    </row>
-    <row r="6" spans="1:23">
+      <c r="S5" s="75"/>
+    </row>
+    <row r="6" spans="1:24">
       <c r="A6" s="2"/>
       <c r="B6" s="18"/>
       <c r="C6" s="19"/>
@@ -2338,9 +2367,9 @@
       <c r="P6" s="17"/>
       <c r="Q6" s="17"/>
       <c r="R6" s="17"/>
-      <c r="S6" s="71"/>
-    </row>
-    <row r="7" spans="1:23">
+      <c r="S6" s="75"/>
+    </row>
+    <row r="7" spans="1:24">
       <c r="A7" s="2"/>
       <c r="B7" s="22"/>
       <c r="C7" s="23"/>
@@ -2359,9 +2388,9 @@
       <c r="P7" s="26"/>
       <c r="Q7" s="26"/>
       <c r="R7" s="26"/>
-      <c r="S7" s="71"/>
-    </row>
-    <row r="8" spans="1:23" ht="15.75" thickBot="1">
+      <c r="S7" s="75"/>
+    </row>
+    <row r="8" spans="1:24" ht="15.75" thickBot="1">
       <c r="A8" s="2"/>
       <c r="B8" s="27"/>
       <c r="C8" s="28"/>
@@ -2380,9 +2409,9 @@
       <c r="P8" s="26"/>
       <c r="Q8" s="26"/>
       <c r="R8" s="26"/>
-      <c r="S8" s="71"/>
-    </row>
-    <row r="9" spans="1:23" ht="15.75" thickBot="1">
+      <c r="S8" s="75"/>
+    </row>
+    <row r="9" spans="1:24" ht="15.75" thickBot="1">
       <c r="A9" s="2"/>
       <c r="B9" s="31" t="s">
         <v>7</v>
@@ -2438,17 +2467,17 @@
       <c r="S9" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="U9" s="78" t="s">
+      <c r="U9" s="68" t="s">
+        <v>352</v>
+      </c>
+      <c r="V9" s="67" t="s">
+        <v>353</v>
+      </c>
+      <c r="W9" s="68" t="s">
         <v>354</v>
       </c>
-      <c r="V9" s="77" t="s">
-        <v>355</v>
-      </c>
-      <c r="W9" s="78" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" ht="24">
+    </row>
+    <row r="10" spans="1:24" ht="24">
       <c r="A10" s="2"/>
       <c r="B10" s="32">
         <f t="shared" ref="B10:B17" si="0">ROW(B10)-ROW($B$9)</f>
@@ -2503,14 +2532,17 @@
       </c>
       <c r="R10" s="34"/>
       <c r="S10" s="57"/>
-      <c r="U10" s="76" t="s">
-        <v>349</v>
+      <c r="U10" s="83" t="s">
+        <v>347</v>
       </c>
       <c r="V10" s="65" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="11" spans="1:23">
+      <c r="X10" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24">
       <c r="A11" s="2"/>
       <c r="B11" s="35">
         <f t="shared" si="0"/>
@@ -2565,14 +2597,17 @@
       </c>
       <c r="R11" s="37"/>
       <c r="S11" s="37"/>
-      <c r="U11" s="64" t="s">
-        <v>334</v>
+      <c r="U11" s="83" t="s">
+        <v>332</v>
       </c>
       <c r="V11" s="65" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="12" spans="1:23" ht="36">
+      <c r="X11" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" ht="36">
       <c r="A12" s="2"/>
       <c r="B12" s="32">
         <f t="shared" si="0"/>
@@ -2627,17 +2662,17 @@
       </c>
       <c r="R12" s="34"/>
       <c r="S12" s="57"/>
-      <c r="U12" s="76" t="s">
-        <v>352</v>
+      <c r="U12" s="83" t="s">
+        <v>350</v>
       </c>
       <c r="V12" s="65" t="s">
         <v>34</v>
       </c>
-      <c r="W12" s="76" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23">
+      <c r="W12" s="66" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24">
       <c r="A13" s="2"/>
       <c r="B13" s="35">
         <f t="shared" si="0"/>
@@ -2692,14 +2727,17 @@
       </c>
       <c r="R13" s="37"/>
       <c r="S13" s="37"/>
-      <c r="U13" s="64" t="s">
-        <v>335</v>
+      <c r="U13" s="83" t="s">
+        <v>333</v>
       </c>
       <c r="V13" s="65" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="14" spans="1:23" ht="24">
+      <c r="X13" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" ht="24">
       <c r="A14" s="2"/>
       <c r="B14" s="32">
         <f t="shared" si="0"/>
@@ -2754,14 +2792,17 @@
       </c>
       <c r="R14" s="34"/>
       <c r="S14" s="57"/>
-      <c r="U14" s="64" t="s">
-        <v>336</v>
+      <c r="U14" s="83" t="s">
+        <v>334</v>
       </c>
       <c r="V14" s="65" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="15" spans="1:23" ht="36">
+      <c r="X14" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" ht="36">
       <c r="A15" s="2"/>
       <c r="B15" s="35">
         <f t="shared" si="0"/>
@@ -2816,17 +2857,20 @@
       </c>
       <c r="R15" s="37"/>
       <c r="S15" s="37"/>
-      <c r="U15" s="79" t="s">
-        <v>358</v>
+      <c r="U15" s="84" t="s">
+        <v>356</v>
       </c>
       <c r="V15" s="65" t="s">
-        <v>357</v>
-      </c>
-      <c r="W15" s="76" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23">
+        <v>355</v>
+      </c>
+      <c r="W15" s="66" t="s">
+        <v>351</v>
+      </c>
+      <c r="X15" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24">
       <c r="A16" s="2"/>
       <c r="B16" s="32">
         <f t="shared" si="0"/>
@@ -2881,14 +2925,17 @@
       </c>
       <c r="R16" s="34"/>
       <c r="S16" s="57"/>
-      <c r="U16" s="64" t="s">
-        <v>337</v>
+      <c r="U16" s="83" t="s">
+        <v>335</v>
       </c>
       <c r="V16" s="65" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="17" spans="1:22" ht="24">
+      <c r="X16" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" ht="24">
       <c r="A17" s="2"/>
       <c r="B17" s="35">
         <f t="shared" si="0"/>
@@ -2943,17 +2990,20 @@
       </c>
       <c r="R17" s="37"/>
       <c r="S17" s="37"/>
-      <c r="U17" s="76" t="s">
-        <v>350</v>
+      <c r="U17" s="83" t="s">
+        <v>348</v>
       </c>
       <c r="V17" s="65" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="18" spans="1:22" ht="24">
+        <v>349</v>
+      </c>
+      <c r="X17" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" ht="24">
       <c r="A18" s="2"/>
       <c r="B18" s="35">
-        <f t="shared" ref="B18:B63" si="3">ROW(B18)-ROW($B$9)</f>
+        <f t="shared" ref="B18:B62" si="3">ROW(B18)-ROW($B$9)</f>
         <v>9</v>
       </c>
       <c r="C18" s="36" t="s">
@@ -2987,7 +3037,7 @@
         <v>3</v>
       </c>
       <c r="M18" s="37">
-        <f t="shared" ref="M18:M63" si="4">L18*5</f>
+        <f t="shared" ref="M18:M62" si="4">L18*5</f>
         <v>15</v>
       </c>
       <c r="N18" s="37">
@@ -3000,19 +3050,22 @@
         <v>8.8000000000000005E-3</v>
       </c>
       <c r="Q18" s="54">
-        <f t="shared" ref="Q18:Q63" si="5">P18*N18</f>
+        <f t="shared" ref="Q18:Q62" si="5">P18*N18</f>
         <v>0.44</v>
       </c>
       <c r="R18" s="37"/>
       <c r="S18" s="37"/>
-      <c r="U18" s="76" t="s">
-        <v>359</v>
+      <c r="U18" s="83" t="s">
+        <v>357</v>
       </c>
       <c r="V18" s="65" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="19" spans="1:22" ht="30">
+      <c r="X18" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" ht="30">
       <c r="A19" s="2"/>
       <c r="B19" s="32">
         <f t="shared" si="3"/>
@@ -3067,14 +3120,17 @@
       </c>
       <c r="R19" s="34"/>
       <c r="S19" s="57"/>
-      <c r="U19" s="79" t="s">
-        <v>360</v>
+      <c r="U19" s="84" t="s">
+        <v>358</v>
       </c>
       <c r="V19" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="20" spans="1:22" ht="36">
+        <v>355</v>
+      </c>
+      <c r="X19" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" ht="36">
       <c r="A20" s="2"/>
       <c r="B20" s="35">
         <f t="shared" si="3"/>
@@ -3129,14 +3185,17 @@
       </c>
       <c r="R20" s="37"/>
       <c r="S20" s="37"/>
-      <c r="U20" s="79" t="s">
-        <v>361</v>
+      <c r="U20" s="84" t="s">
+        <v>359</v>
       </c>
       <c r="V20" s="65" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="21" spans="1:22" ht="60">
+        <v>360</v>
+      </c>
+      <c r="X20" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" ht="60">
       <c r="A21" s="2"/>
       <c r="B21" s="32">
         <f t="shared" si="3"/>
@@ -3189,14 +3248,20 @@
       </c>
       <c r="R21" s="34"/>
       <c r="S21" s="57"/>
-      <c r="U21" s="79" t="s">
-        <v>367</v>
+      <c r="U21" s="84" t="s">
+        <v>365</v>
       </c>
       <c r="V21" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="22" spans="1:22" ht="60">
+        <v>355</v>
+      </c>
+      <c r="W21" s="82" t="s">
+        <v>371</v>
+      </c>
+      <c r="X21" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" ht="60">
       <c r="A22" s="2"/>
       <c r="B22" s="35">
         <f t="shared" si="3"/>
@@ -3249,14 +3314,20 @@
       </c>
       <c r="R22" s="37"/>
       <c r="S22" s="37"/>
-      <c r="U22">
+      <c r="U22" s="83">
         <v>1206180000</v>
       </c>
       <c r="V22" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="23" spans="1:22" ht="24">
+        <v>355</v>
+      </c>
+      <c r="W22" s="82" t="s">
+        <v>371</v>
+      </c>
+      <c r="X22" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" ht="24">
       <c r="A23" s="2"/>
       <c r="B23" s="32">
         <f t="shared" si="3"/>
@@ -3312,8 +3383,11 @@
       <c r="V23" s="64" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="24" spans="1:22" ht="48">
+      <c r="X23" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" ht="48">
       <c r="A24" s="2"/>
       <c r="B24" s="35">
         <f t="shared" si="3"/>
@@ -3366,14 +3440,14 @@
       </c>
       <c r="R24" s="37"/>
       <c r="S24" s="37"/>
-      <c r="U24" s="79" t="s">
-        <v>369</v>
+      <c r="U24" s="84" t="s">
+        <v>367</v>
       </c>
       <c r="V24" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="25" spans="1:22">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="25" spans="1:24">
       <c r="A25" s="2"/>
       <c r="B25" s="32">
         <f t="shared" si="3"/>
@@ -3426,14 +3500,14 @@
       </c>
       <c r="R25" s="34"/>
       <c r="S25" s="57"/>
-      <c r="U25" s="76" t="s">
-        <v>370</v>
+      <c r="U25" s="83" t="s">
+        <v>368</v>
       </c>
       <c r="V25" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="26" spans="1:22" ht="30">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="26" spans="1:24" ht="30">
       <c r="A26" s="2"/>
       <c r="B26" s="35">
         <f t="shared" si="3"/>
@@ -3486,14 +3560,14 @@
       </c>
       <c r="R26" s="37"/>
       <c r="S26" s="37"/>
-      <c r="U26" s="79" t="s">
-        <v>368</v>
+      <c r="U26" s="84" t="s">
+        <v>366</v>
       </c>
       <c r="V26" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="27" spans="1:22" ht="48">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="27" spans="1:24" ht="48">
       <c r="A27" s="2"/>
       <c r="B27" s="32">
         <f t="shared" si="3"/>
@@ -3549,14 +3623,14 @@
         <v>130</v>
       </c>
       <c r="S27" s="58"/>
-      <c r="U27" s="81" t="s">
+      <c r="U27" s="69" t="s">
         <v>129</v>
       </c>
       <c r="V27" s="64" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="1:22" ht="24">
+    <row r="28" spans="1:24" ht="24">
       <c r="A28" s="2"/>
       <c r="B28" s="35">
         <f t="shared" si="3"/>
@@ -3611,14 +3685,14 @@
       </c>
       <c r="R28" s="37"/>
       <c r="S28" s="37"/>
-      <c r="U28" s="76" t="s">
-        <v>364</v>
+      <c r="U28" s="66" t="s">
+        <v>362</v>
       </c>
       <c r="V28" s="64" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:22" ht="36">
+    <row r="29" spans="1:24" ht="36">
       <c r="A29" s="2"/>
       <c r="B29" s="32">
         <f t="shared" si="3"/>
@@ -3674,14 +3748,14 @@
         <v>130</v>
       </c>
       <c r="S29" s="58"/>
-      <c r="U29" s="81" t="s">
+      <c r="U29" s="69" t="s">
         <v>129</v>
       </c>
       <c r="V29" s="64" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:22" ht="48">
+    <row r="30" spans="1:24" ht="48">
       <c r="A30" s="2"/>
       <c r="B30" s="35">
         <f t="shared" si="3"/>
@@ -3736,14 +3810,20 @@
       </c>
       <c r="R30" s="37"/>
       <c r="S30" s="37"/>
-      <c r="U30">
+      <c r="U30" s="83">
         <v>691137710002</v>
       </c>
       <c r="V30" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="31" spans="1:22" ht="36">
+        <v>355</v>
+      </c>
+      <c r="W30" s="82" t="s">
+        <v>371</v>
+      </c>
+      <c r="X30" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="31" spans="1:24" ht="36">
       <c r="A31" s="2"/>
       <c r="B31" s="32">
         <f t="shared" si="3"/>
@@ -3801,8 +3881,11 @@
       <c r="V31" s="64" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="32" spans="1:22">
+      <c r="X31" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="32" spans="1:24">
       <c r="A32" s="2"/>
       <c r="B32" s="35">
         <f t="shared" si="3"/>
@@ -3857,14 +3940,20 @@
       </c>
       <c r="R32" s="37"/>
       <c r="S32" s="37"/>
-      <c r="U32" s="76" t="s">
+      <c r="U32" s="83" t="s">
+        <v>369</v>
+      </c>
+      <c r="V32" s="65" t="s">
+        <v>355</v>
+      </c>
+      <c r="W32" s="82" t="s">
         <v>371</v>
       </c>
-      <c r="V32" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="33" spans="1:22" ht="24">
+      <c r="X32" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="33" spans="1:24" ht="24">
       <c r="A33" s="2"/>
       <c r="B33" s="32">
         <f t="shared" si="3"/>
@@ -3919,14 +4008,17 @@
       </c>
       <c r="R33" s="34"/>
       <c r="S33" s="57"/>
-      <c r="U33" s="76" t="s">
-        <v>372</v>
+      <c r="U33" s="83" t="s">
+        <v>370</v>
       </c>
       <c r="V33" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="34" spans="1:22" ht="24">
+        <v>355</v>
+      </c>
+      <c r="X33" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="34" spans="1:24" ht="24">
       <c r="A34" s="2"/>
       <c r="B34" s="35">
         <f t="shared" si="3"/>
@@ -3981,14 +4073,14 @@
       </c>
       <c r="R34" s="37"/>
       <c r="S34" s="37"/>
-      <c r="U34" s="76" t="s">
-        <v>364</v>
+      <c r="U34" s="66" t="s">
+        <v>362</v>
       </c>
       <c r="V34" s="64" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:22" ht="36">
+    <row r="35" spans="1:24" ht="36">
       <c r="A35" s="2"/>
       <c r="B35" s="32">
         <f t="shared" si="3"/>
@@ -4043,14 +4135,14 @@
       </c>
       <c r="R35" s="34"/>
       <c r="S35" s="57"/>
-      <c r="U35" s="76" t="s">
-        <v>364</v>
+      <c r="U35" s="66" t="s">
+        <v>362</v>
       </c>
       <c r="V35" s="64" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:22" ht="36">
+    <row r="36" spans="1:24" ht="36">
       <c r="A36" s="2"/>
       <c r="B36" s="35">
         <f t="shared" si="3"/>
@@ -4105,14 +4197,14 @@
       </c>
       <c r="R36" s="37"/>
       <c r="S36" s="37"/>
-      <c r="U36" s="76" t="s">
-        <v>364</v>
+      <c r="U36" s="66" t="s">
+        <v>362</v>
       </c>
       <c r="V36" s="64" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:22" ht="25.5">
+    <row r="37" spans="1:24" ht="25.5">
       <c r="A37" s="2"/>
       <c r="B37" s="32">
         <f t="shared" si="3"/>
@@ -4171,7 +4263,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="38" spans="1:22">
+    <row r="38" spans="1:24">
       <c r="A38" s="2"/>
       <c r="B38" s="35">
         <f t="shared" si="3"/>
@@ -4226,14 +4318,14 @@
       </c>
       <c r="R38" s="37"/>
       <c r="S38" s="37"/>
-      <c r="U38" s="64" t="s">
-        <v>338</v>
+      <c r="U38" s="83" t="s">
+        <v>336</v>
       </c>
       <c r="V38" s="65" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="39" spans="1:22">
+    <row r="39" spans="1:24">
       <c r="A39" s="2"/>
       <c r="B39" s="32">
         <f t="shared" si="3"/>
@@ -4288,14 +4380,14 @@
       </c>
       <c r="R39" s="34"/>
       <c r="S39" s="57"/>
-      <c r="U39" s="64" t="s">
-        <v>339</v>
+      <c r="U39" s="83" t="s">
+        <v>337</v>
       </c>
       <c r="V39" s="65" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="40" spans="1:22">
+    <row r="40" spans="1:24">
       <c r="A40" s="2"/>
       <c r="B40" s="35">
         <f t="shared" si="3"/>
@@ -4350,14 +4442,14 @@
       </c>
       <c r="R40" s="37"/>
       <c r="S40" s="37"/>
-      <c r="U40" s="64" t="s">
-        <v>340</v>
+      <c r="U40" s="83" t="s">
+        <v>338</v>
       </c>
       <c r="V40" s="65" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:22">
+    <row r="41" spans="1:24">
       <c r="A41" s="2"/>
       <c r="B41" s="32">
         <f t="shared" si="3"/>
@@ -4412,14 +4504,14 @@
       </c>
       <c r="R41" s="34"/>
       <c r="S41" s="57"/>
-      <c r="U41" s="64" t="s">
-        <v>341</v>
+      <c r="U41" s="83" t="s">
+        <v>339</v>
       </c>
       <c r="V41" s="65" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="42" spans="1:22">
+    <row r="42" spans="1:24">
       <c r="A42" s="2"/>
       <c r="B42" s="35">
         <f t="shared" si="3"/>
@@ -4474,14 +4566,14 @@
       </c>
       <c r="R42" s="37"/>
       <c r="S42" s="37"/>
-      <c r="U42" s="64" t="s">
-        <v>342</v>
+      <c r="U42" s="83" t="s">
+        <v>340</v>
       </c>
       <c r="V42" s="65" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="43" spans="1:22">
+    <row r="43" spans="1:24">
       <c r="A43" s="2"/>
       <c r="B43" s="32">
         <f t="shared" si="3"/>
@@ -4536,14 +4628,14 @@
       </c>
       <c r="R43" s="34"/>
       <c r="S43" s="57"/>
-      <c r="U43" s="64" t="s">
-        <v>343</v>
+      <c r="U43" s="83" t="s">
+        <v>341</v>
       </c>
       <c r="V43" s="65" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:22">
+    <row r="44" spans="1:24">
       <c r="A44" s="2"/>
       <c r="B44" s="35">
         <f t="shared" si="3"/>
@@ -4598,14 +4690,14 @@
       </c>
       <c r="R44" s="37"/>
       <c r="S44" s="37"/>
-      <c r="U44" s="64" t="s">
-        <v>344</v>
+      <c r="U44" s="83" t="s">
+        <v>342</v>
       </c>
       <c r="V44" s="65" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="45" spans="1:22">
+    <row r="45" spans="1:24">
       <c r="A45" s="2"/>
       <c r="B45" s="32">
         <f t="shared" si="3"/>
@@ -4660,14 +4752,14 @@
       </c>
       <c r="R45" s="34"/>
       <c r="S45" s="57"/>
-      <c r="U45" s="64" t="s">
-        <v>345</v>
+      <c r="U45" s="83" t="s">
+        <v>343</v>
       </c>
       <c r="V45" s="65" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="46" spans="1:22">
+    <row r="46" spans="1:24">
       <c r="A46" s="2"/>
       <c r="B46" s="35">
         <f t="shared" si="3"/>
@@ -4722,14 +4814,14 @@
       </c>
       <c r="R46" s="37"/>
       <c r="S46" s="37"/>
-      <c r="U46" s="64" t="s">
-        <v>346</v>
+      <c r="U46" s="83" t="s">
+        <v>344</v>
       </c>
       <c r="V46" s="65" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="47" spans="1:22">
+    <row r="47" spans="1:24">
       <c r="A47" s="2"/>
       <c r="B47" s="32">
         <f t="shared" si="3"/>
@@ -4784,14 +4876,14 @@
       </c>
       <c r="R47" s="34"/>
       <c r="S47" s="57"/>
-      <c r="U47" s="64" t="s">
-        <v>347</v>
+      <c r="U47" s="83" t="s">
+        <v>345</v>
       </c>
       <c r="V47" s="65" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="48" spans="1:22">
+    <row r="48" spans="1:24">
       <c r="A48" s="2"/>
       <c r="B48" s="35">
         <f t="shared" si="3"/>
@@ -4846,14 +4938,14 @@
       </c>
       <c r="R48" s="37"/>
       <c r="S48" s="37"/>
-      <c r="U48" s="64" t="s">
-        <v>348</v>
+      <c r="U48" s="83" t="s">
+        <v>346</v>
       </c>
       <c r="V48" s="65" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="49" spans="1:22" ht="24">
+    <row r="49" spans="1:24" ht="24">
       <c r="A49" s="2"/>
       <c r="B49" s="32">
         <f t="shared" si="3"/>
@@ -4908,11 +5000,17 @@
       </c>
       <c r="R49" s="34"/>
       <c r="S49" s="57"/>
-      <c r="V49" s="64" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="50" spans="1:22" ht="24">
+      <c r="U49" s="81" t="s">
+        <v>373</v>
+      </c>
+      <c r="V49" s="65" t="s">
+        <v>355</v>
+      </c>
+      <c r="W49" s="82" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="50" spans="1:24" ht="24">
       <c r="A50" s="2"/>
       <c r="B50" s="35">
         <f t="shared" si="3"/>
@@ -4971,7 +5069,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="51" spans="1:22" ht="24">
+    <row r="51" spans="1:24" ht="24">
       <c r="A51" s="2"/>
       <c r="B51" s="32">
         <f t="shared" si="3"/>
@@ -5026,11 +5124,15 @@
       </c>
       <c r="R51" s="34"/>
       <c r="S51" s="57"/>
-      <c r="V51" s="64" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="52" spans="1:22" ht="36">
+      <c r="U51" s="80" t="s">
+        <v>362</v>
+      </c>
+      <c r="V51" s="65"/>
+      <c r="W51" s="82" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="52" spans="1:24" ht="36">
       <c r="A52" s="2"/>
       <c r="B52" s="35">
         <f t="shared" si="3"/>
@@ -5085,11 +5187,14 @@
       </c>
       <c r="R52" s="37"/>
       <c r="S52" s="37"/>
+      <c r="U52" s="82" t="s">
+        <v>362</v>
+      </c>
       <c r="V52" s="64" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="53" spans="1:22" ht="36">
+    <row r="53" spans="1:24" ht="36">
       <c r="A53" s="2"/>
       <c r="B53" s="32">
         <f t="shared" si="3"/>
@@ -5148,7 +5253,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="54" spans="1:22">
+    <row r="54" spans="1:24">
       <c r="A54" s="2"/>
       <c r="B54" s="35">
         <f t="shared" si="3"/>
@@ -5203,11 +5308,14 @@
       </c>
       <c r="R54" s="37"/>
       <c r="S54" s="37"/>
+      <c r="U54" s="82" t="s">
+        <v>362</v>
+      </c>
       <c r="V54" s="64" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="55" spans="1:22">
+    <row r="55" spans="1:24">
       <c r="A55" s="2"/>
       <c r="B55" s="32">
         <f t="shared" si="3"/>
@@ -5266,7 +5374,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="56" spans="1:22" ht="24">
+    <row r="56" spans="1:24" ht="24">
       <c r="A56" s="2"/>
       <c r="B56" s="35">
         <f t="shared" si="3"/>
@@ -5321,14 +5429,17 @@
       </c>
       <c r="R56" s="37"/>
       <c r="S56" s="37"/>
-      <c r="U56" s="76" t="s">
-        <v>365</v>
+      <c r="U56" s="83" t="s">
+        <v>363</v>
       </c>
       <c r="V56" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="57" spans="1:22">
+        <v>355</v>
+      </c>
+      <c r="X56" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="57" spans="1:24">
       <c r="A57" s="2"/>
       <c r="B57" s="32">
         <f t="shared" si="3"/>
@@ -5383,14 +5494,20 @@
       </c>
       <c r="R57" s="34"/>
       <c r="S57" s="57"/>
-      <c r="U57" s="80" t="s">
-        <v>363</v>
+      <c r="U57" s="85" t="s">
+        <v>361</v>
       </c>
       <c r="V57" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="58" spans="1:22" ht="24">
+        <v>355</v>
+      </c>
+      <c r="W57" s="82" t="s">
+        <v>372</v>
+      </c>
+      <c r="X57" s="82" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="58" spans="1:24" ht="24">
       <c r="A58" s="2"/>
       <c r="B58" s="35">
         <f t="shared" si="3"/>
@@ -5445,14 +5562,14 @@
       </c>
       <c r="R58" s="37"/>
       <c r="S58" s="37"/>
-      <c r="U58" s="76" t="s">
-        <v>364</v>
+      <c r="U58" s="66" t="s">
+        <v>362</v>
       </c>
       <c r="V58" s="64" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="59" spans="1:22">
+    <row r="59" spans="1:24">
       <c r="A59" s="2"/>
       <c r="B59" s="32">
         <f t="shared" si="3"/>
@@ -5507,14 +5624,14 @@
       </c>
       <c r="R59" s="34"/>
       <c r="S59" s="57"/>
-      <c r="U59" s="76" t="s">
-        <v>366</v>
+      <c r="U59" s="66" t="s">
+        <v>364</v>
       </c>
       <c r="V59" s="64" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="60" spans="1:22" ht="36">
+    <row r="60" spans="1:24" ht="36">
       <c r="A60" s="2"/>
       <c r="B60" s="32">
         <f t="shared" si="3"/>
@@ -5573,10 +5690,10 @@
         <v>1282360000</v>
       </c>
       <c r="V60" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="61" spans="1:22" ht="36">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="61" spans="1:24" ht="36">
       <c r="A61" s="2"/>
       <c r="B61" s="32">
         <f t="shared" si="3"/>
@@ -5635,10 +5752,10 @@
         <v>1206180000</v>
       </c>
       <c r="V61" s="65" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="62" spans="1:22" ht="24">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="62" spans="1:24" ht="24.75" thickBot="1">
       <c r="A62" s="2"/>
       <c r="B62" s="32">
         <f t="shared" si="3"/>
@@ -5693,128 +5810,72 @@
       </c>
       <c r="R62" s="34"/>
       <c r="S62" s="57"/>
+      <c r="U62" s="82" t="s">
+        <v>362</v>
+      </c>
       <c r="V62" s="64" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="63" spans="1:22" ht="36">
+    <row r="63" spans="1:24" ht="19.5" thickBot="1">
       <c r="A63" s="2"/>
-      <c r="B63" s="32">
-        <f t="shared" si="3"/>
-        <v>54</v>
-      </c>
-      <c r="C63" s="33" t="s">
-        <v>320</v>
-      </c>
-      <c r="D63" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="E63" s="34" t="s">
-        <v>333</v>
-      </c>
-      <c r="F63" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="G63" s="34" t="s">
-        <v>332</v>
-      </c>
-      <c r="H63" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="I63" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J63" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="K63" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="L63" s="34">
-        <v>1</v>
-      </c>
-      <c r="M63" s="34">
-        <f t="shared" si="4"/>
-        <v>5</v>
-      </c>
-      <c r="N63" s="34">
-        <v>5</v>
-      </c>
-      <c r="O63" s="51" t="s">
-        <v>282</v>
-      </c>
-      <c r="P63" s="52">
-        <v>2</v>
-      </c>
-      <c r="Q63" s="52">
-        <f t="shared" si="5"/>
-        <v>10</v>
-      </c>
-      <c r="R63" s="34"/>
-      <c r="S63" s="57"/>
-      <c r="V63" s="64" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="64" spans="1:22" ht="18.75">
+      <c r="B63" s="41"/>
+      <c r="C63" s="42"/>
+      <c r="D63" s="43"/>
+      <c r="E63" s="44"/>
+      <c r="F63" s="45"/>
+      <c r="G63" s="46"/>
+      <c r="H63" s="45"/>
+      <c r="I63" s="46"/>
+      <c r="J63" s="45"/>
+      <c r="K63" s="46"/>
+      <c r="L63" s="46"/>
+      <c r="M63" s="46"/>
+      <c r="N63" s="72" t="s">
+        <v>318</v>
+      </c>
+      <c r="O63" s="73"/>
+      <c r="P63" s="73"/>
+      <c r="Q63" s="59">
+        <f>SUM(Q10:Q62)</f>
+        <v>121.5672</v>
+      </c>
+      <c r="R63" s="76"/>
+      <c r="S63" s="77"/>
+    </row>
+    <row r="64" spans="1:24" ht="18.75">
       <c r="A64" s="2"/>
-      <c r="B64" s="41"/>
-      <c r="C64" s="42"/>
-      <c r="D64" s="43"/>
-      <c r="E64" s="44"/>
-      <c r="F64" s="45"/>
-      <c r="G64" s="46"/>
-      <c r="H64" s="45"/>
-      <c r="I64" s="46"/>
-      <c r="J64" s="45"/>
-      <c r="K64" s="46"/>
-      <c r="L64" s="46"/>
-      <c r="M64" s="46"/>
-      <c r="N64" s="68" t="s">
-        <v>318</v>
-      </c>
-      <c r="O64" s="69"/>
-      <c r="P64" s="69"/>
-      <c r="Q64" s="59">
-        <f>SUM(Q10:Q63)</f>
-        <v>131.56720000000001</v>
-      </c>
-      <c r="R64" s="72"/>
-      <c r="S64" s="73"/>
-    </row>
-    <row r="65" spans="1:19" ht="18.75">
-      <c r="A65" s="2"/>
-      <c r="B65" s="47"/>
-      <c r="C65" s="48"/>
-      <c r="D65" s="49"/>
-      <c r="E65" s="50"/>
-      <c r="F65" s="50"/>
-      <c r="G65" s="50"/>
-      <c r="H65" s="50"/>
-      <c r="I65" s="50"/>
-      <c r="J65" s="50"/>
-      <c r="K65" s="50"/>
-      <c r="L65" s="50"/>
-      <c r="M65" s="50"/>
-      <c r="N65" s="68" t="s">
+      <c r="B64" s="47"/>
+      <c r="C64" s="48"/>
+      <c r="D64" s="49"/>
+      <c r="E64" s="50"/>
+      <c r="F64" s="50"/>
+      <c r="G64" s="50"/>
+      <c r="H64" s="50"/>
+      <c r="I64" s="50"/>
+      <c r="J64" s="50"/>
+      <c r="K64" s="50"/>
+      <c r="L64" s="50"/>
+      <c r="M64" s="50"/>
+      <c r="N64" s="72" t="s">
         <v>319</v>
       </c>
-      <c r="O65" s="69"/>
-      <c r="P65" s="69"/>
-      <c r="Q65" s="60">
-        <f>Q64/5</f>
-        <v>26.313440000000003</v>
-      </c>
-      <c r="R65" s="74"/>
-      <c r="S65" s="75"/>
+      <c r="O64" s="73"/>
+      <c r="P64" s="73"/>
+      <c r="Q64" s="60">
+        <f>Q63/5</f>
+        <v>24.31344</v>
+      </c>
+      <c r="R64" s="78"/>
+      <c r="S64" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
+    <mergeCell ref="N63:P63"/>
     <mergeCell ref="N64:P64"/>
-    <mergeCell ref="N65:P65"/>
     <mergeCell ref="S3:S8"/>
-    <mergeCell ref="R64:S65"/>
+    <mergeCell ref="R63:S64"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O10" r:id="rId1"/>
@@ -5868,41 +5929,41 @@
     <hyperlink ref="O60" r:id="rId49"/>
     <hyperlink ref="O61" r:id="rId50"/>
     <hyperlink ref="O62" r:id="rId51"/>
-    <hyperlink ref="O63" r:id="rId52"/>
-    <hyperlink ref="V11" r:id="rId53"/>
-    <hyperlink ref="V13" r:id="rId54"/>
-    <hyperlink ref="V14" r:id="rId55"/>
-    <hyperlink ref="V16" r:id="rId56"/>
-    <hyperlink ref="V38" r:id="rId57"/>
-    <hyperlink ref="V39" r:id="rId58"/>
-    <hyperlink ref="V40" r:id="rId59"/>
-    <hyperlink ref="V41" r:id="rId60"/>
-    <hyperlink ref="V42" r:id="rId61"/>
-    <hyperlink ref="V43" r:id="rId62"/>
-    <hyperlink ref="V44" r:id="rId63"/>
-    <hyperlink ref="V45" r:id="rId64"/>
-    <hyperlink ref="V46" r:id="rId65"/>
-    <hyperlink ref="V47" r:id="rId66"/>
-    <hyperlink ref="V48" r:id="rId67"/>
-    <hyperlink ref="V10" r:id="rId68"/>
-    <hyperlink ref="V17" r:id="rId69"/>
-    <hyperlink ref="V12" r:id="rId70"/>
-    <hyperlink ref="V15" r:id="rId71"/>
-    <hyperlink ref="V18" r:id="rId72"/>
-    <hyperlink ref="V19" r:id="rId73"/>
-    <hyperlink ref="V20" r:id="rId74"/>
-    <hyperlink ref="V57" r:id="rId75"/>
-    <hyperlink ref="V56" r:id="rId76"/>
-    <hyperlink ref="V21" r:id="rId77"/>
-    <hyperlink ref="V60" r:id="rId78"/>
-    <hyperlink ref="V22" r:id="rId79"/>
-    <hyperlink ref="V61" r:id="rId80"/>
-    <hyperlink ref="V26" r:id="rId81"/>
-    <hyperlink ref="V24" r:id="rId82"/>
-    <hyperlink ref="V25" r:id="rId83"/>
-    <hyperlink ref="V30" r:id="rId84"/>
-    <hyperlink ref="V32" r:id="rId85"/>
-    <hyperlink ref="V33" r:id="rId86"/>
+    <hyperlink ref="V11" r:id="rId52"/>
+    <hyperlink ref="V13" r:id="rId53"/>
+    <hyperlink ref="V14" r:id="rId54"/>
+    <hyperlink ref="V16" r:id="rId55"/>
+    <hyperlink ref="V38" r:id="rId56"/>
+    <hyperlink ref="V39" r:id="rId57"/>
+    <hyperlink ref="V40" r:id="rId58"/>
+    <hyperlink ref="V41" r:id="rId59"/>
+    <hyperlink ref="V42" r:id="rId60"/>
+    <hyperlink ref="V43" r:id="rId61"/>
+    <hyperlink ref="V44" r:id="rId62"/>
+    <hyperlink ref="V45" r:id="rId63"/>
+    <hyperlink ref="V46" r:id="rId64"/>
+    <hyperlink ref="V47" r:id="rId65"/>
+    <hyperlink ref="V48" r:id="rId66"/>
+    <hyperlink ref="V10" r:id="rId67"/>
+    <hyperlink ref="V17" r:id="rId68"/>
+    <hyperlink ref="V12" r:id="rId69"/>
+    <hyperlink ref="V15" r:id="rId70"/>
+    <hyperlink ref="V18" r:id="rId71"/>
+    <hyperlink ref="V19" r:id="rId72"/>
+    <hyperlink ref="V20" r:id="rId73"/>
+    <hyperlink ref="V57" r:id="rId74"/>
+    <hyperlink ref="V56" r:id="rId75"/>
+    <hyperlink ref="V21" r:id="rId76"/>
+    <hyperlink ref="V60" r:id="rId77"/>
+    <hyperlink ref="V22" r:id="rId78"/>
+    <hyperlink ref="V61" r:id="rId79"/>
+    <hyperlink ref="V26" r:id="rId80"/>
+    <hyperlink ref="V24" r:id="rId81"/>
+    <hyperlink ref="V25" r:id="rId82"/>
+    <hyperlink ref="V30" r:id="rId83"/>
+    <hyperlink ref="V32" r:id="rId84"/>
+    <hyperlink ref="V33" r:id="rId85"/>
+    <hyperlink ref="V49" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
#8 PCB Placement and routing in progress.
</commit_message>
<xml_diff>
--- a/Design-Files/MotorDriver-v1.0/Deliverables/BOM/eSpark BOM.xlsx
+++ b/Design-Files/MotorDriver-v1.0/Deliverables/BOM/eSpark BOM.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="372">
   <si>
     <t>Component list</t>
   </si>
@@ -1138,6 +1138,9 @@
   </si>
   <si>
     <t>Updated in PCB</t>
+  </si>
+  <si>
+    <t>IF-6-24</t>
   </si>
 </sst>
 </file>
@@ -3401,7 +3404,7 @@
       <c r="U23" s="73" t="s">
         <v>363</v>
       </c>
-      <c r="V23" s="64" t="s">
+      <c r="V23" s="65" t="s">
         <v>34</v>
       </c>
       <c r="X23" s="79" t="s">
@@ -3656,9 +3659,7 @@
       <c r="U27" s="69" t="s">
         <v>129</v>
       </c>
-      <c r="V27" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V27" s="64"/>
     </row>
     <row r="28" spans="1:25" ht="24">
       <c r="A28" s="2"/>
@@ -3718,9 +3719,7 @@
       <c r="U28" s="66" t="s">
         <v>361</v>
       </c>
-      <c r="V28" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V28" s="64"/>
     </row>
     <row r="29" spans="1:25" ht="36">
       <c r="A29" s="2"/>
@@ -3781,9 +3780,7 @@
       <c r="U29" s="69" t="s">
         <v>129</v>
       </c>
-      <c r="V29" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V29" s="64"/>
     </row>
     <row r="30" spans="1:25" ht="48">
       <c r="A30" s="2"/>
@@ -3911,9 +3908,7 @@
       <c r="U31" s="79" t="s">
         <v>361</v>
       </c>
-      <c r="V31" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V31" s="64"/>
       <c r="X31" s="79"/>
     </row>
     <row r="32" spans="1:25">
@@ -4103,9 +4098,7 @@
       <c r="U34" s="66" t="s">
         <v>361</v>
       </c>
-      <c r="V34" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V34" s="64"/>
     </row>
     <row r="35" spans="1:24" ht="36">
       <c r="A35" s="2"/>
@@ -4165,9 +4158,7 @@
       <c r="U35" s="66" t="s">
         <v>361</v>
       </c>
-      <c r="V35" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V35" s="64"/>
     </row>
     <row r="36" spans="1:24" ht="36">
       <c r="A36" s="2"/>
@@ -4227,9 +4218,7 @@
       <c r="U36" s="66" t="s">
         <v>361</v>
       </c>
-      <c r="V36" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V36" s="64"/>
     </row>
     <row r="37" spans="1:24" ht="25.5">
       <c r="A37" s="2"/>
@@ -4289,9 +4278,7 @@
       <c r="U37" s="79" t="s">
         <v>361</v>
       </c>
-      <c r="V37" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V37" s="64"/>
     </row>
     <row r="38" spans="1:24">
       <c r="A38" s="2"/>
@@ -5132,9 +5119,7 @@
       </c>
       <c r="R50" s="37"/>
       <c r="S50" s="37"/>
-      <c r="V50" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V50" s="64"/>
     </row>
     <row r="51" spans="1:25" ht="24">
       <c r="A51" s="2"/>
@@ -5195,9 +5180,7 @@
         <v>361</v>
       </c>
       <c r="V51" s="65"/>
-      <c r="W51" s="71" t="s">
-        <v>367</v>
-      </c>
+      <c r="W51" s="71"/>
     </row>
     <row r="52" spans="1:25" ht="36">
       <c r="A52" s="2"/>
@@ -5257,9 +5240,7 @@
       <c r="U52" s="71" t="s">
         <v>361</v>
       </c>
-      <c r="V52" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V52" s="64"/>
     </row>
     <row r="53" spans="1:25" ht="36">
       <c r="A53" s="2"/>
@@ -5316,8 +5297,11 @@
       </c>
       <c r="R53" s="34"/>
       <c r="S53" s="57"/>
-      <c r="V53" s="64" t="s">
-        <v>34</v>
+      <c r="U53" t="s">
+        <v>371</v>
+      </c>
+      <c r="V53" s="65" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="54" spans="1:25">
@@ -5378,9 +5362,7 @@
       <c r="U54" s="71" t="s">
         <v>361</v>
       </c>
-      <c r="V54" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V54" s="64"/>
     </row>
     <row r="55" spans="1:25">
       <c r="A55" s="2"/>
@@ -5440,9 +5422,7 @@
       <c r="U55" s="77" t="s">
         <v>361</v>
       </c>
-      <c r="V55" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V55" s="64"/>
     </row>
     <row r="56" spans="1:25" ht="24">
       <c r="A56" s="2"/>
@@ -5634,9 +5614,7 @@
       <c r="U58" s="66" t="s">
         <v>361</v>
       </c>
-      <c r="V58" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V58" s="64"/>
     </row>
     <row r="59" spans="1:25">
       <c r="A59" s="2"/>
@@ -5696,9 +5674,7 @@
       <c r="U59" s="66" t="s">
         <v>361</v>
       </c>
-      <c r="V59" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V59" s="64"/>
     </row>
     <row r="60" spans="1:25" ht="36">
       <c r="A60" s="2"/>
@@ -5878,9 +5854,7 @@
       <c r="U62" s="71" t="s">
         <v>361</v>
       </c>
-      <c r="V62" s="64" t="s">
-        <v>34</v>
-      </c>
+      <c r="V62" s="64"/>
     </row>
     <row r="63" spans="1:25" ht="19.5" thickBot="1">
       <c r="A63" s="2"/>
@@ -6027,9 +6001,11 @@
     <hyperlink ref="V49" r:id="rId82"/>
     <hyperlink ref="V26" r:id="rId83"/>
     <hyperlink ref="V30" r:id="rId84"/>
+    <hyperlink ref="V23" r:id="rId85"/>
+    <hyperlink ref="V53" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId85"/>
-  <drawing r:id="rId86"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId87"/>
+  <drawing r:id="rId88"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#10 Alternate Part Number added
</commit_message>
<xml_diff>
--- a/Design-Files/MotorDriver-v1.0/Deliverables/BOM/eSpark BOM.xlsx
+++ b/Design-Files/MotorDriver-v1.0/Deliverables/BOM/eSpark BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\hasanmehmood-motordriver\Design-Files\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\hasanmehmood-motordriver\Design-Files\MotorDriver-v1.0\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="335">
   <si>
     <t>Component list</t>
   </si>
@@ -426,9 +426,6 @@
     <t>0PTF0078P</t>
   </si>
   <si>
-    <t>C2760101</t>
-  </si>
-  <si>
     <t>Female Header</t>
   </si>
   <si>
@@ -1021,6 +1018,12 @@
   </si>
   <si>
     <t>High sensitivity wireless remote control receiving module RXB61 multiple frequency 315M.433MHZ</t>
+  </si>
+  <si>
+    <t>PTF-77</t>
+  </si>
+  <si>
+    <t>C717030</t>
   </si>
 </sst>
 </file>
@@ -3298,10 +3301,10 @@
         <v>89</v>
       </c>
       <c r="I28" s="37" t="s">
-        <v>31</v>
+        <v>333</v>
       </c>
       <c r="J28" s="37" t="s">
-        <v>135</v>
+        <v>334</v>
       </c>
       <c r="K28" s="37" t="s">
         <v>31</v>
@@ -3314,17 +3317,17 @@
         <v>5</v>
       </c>
       <c r="N28" s="37">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O28" s="53" t="s">
         <v>34</v>
       </c>
       <c r="P28" s="54">
-        <v>0.80349999999999999</v>
+        <v>0.13689999999999999</v>
       </c>
       <c r="Q28" s="54">
         <f t="shared" si="5"/>
-        <v>4.8209999999999997</v>
+        <v>1.369</v>
       </c>
       <c r="R28" s="37"/>
       <c r="S28" s="37"/>
@@ -3336,28 +3339,28 @@
         <v>20</v>
       </c>
       <c r="C29" s="40" t="s">
+        <v>135</v>
+      </c>
+      <c r="D29" s="39" t="s">
         <v>136</v>
       </c>
-      <c r="D29" s="39" t="s">
+      <c r="E29" s="39" t="s">
         <v>137</v>
       </c>
-      <c r="E29" s="39" t="s">
+      <c r="F29" s="39" t="s">
         <v>138</v>
       </c>
-      <c r="F29" s="39" t="s">
+      <c r="G29" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="G29" s="39" t="s">
+      <c r="H29" s="39" t="s">
         <v>140</v>
       </c>
-      <c r="H29" s="39" t="s">
-        <v>141</v>
-      </c>
       <c r="I29" s="39" t="s">
         <v>31</v>
       </c>
       <c r="J29" s="39" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K29" s="39" t="s">
         <v>129</v>
@@ -3396,16 +3399,16 @@
         <v>97</v>
       </c>
       <c r="D30" s="37" t="s">
+        <v>141</v>
+      </c>
+      <c r="E30" s="37" t="s">
         <v>142</v>
-      </c>
-      <c r="E30" s="37" t="s">
-        <v>143</v>
       </c>
       <c r="F30" s="37" t="s">
         <v>28</v>
       </c>
       <c r="G30" s="37" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H30" s="37" t="s">
         <v>101</v>
@@ -3414,7 +3417,7 @@
         <v>31</v>
       </c>
       <c r="J30" s="37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K30" s="37" t="s">
         <v>31</v>
@@ -3449,28 +3452,28 @@
         <v>22</v>
       </c>
       <c r="C31" s="33" t="s">
+        <v>145</v>
+      </c>
+      <c r="D31" s="34" t="s">
         <v>146</v>
       </c>
-      <c r="D31" s="34" t="s">
+      <c r="E31" s="34" t="s">
         <v>147</v>
-      </c>
-      <c r="E31" s="34" t="s">
-        <v>148</v>
       </c>
       <c r="F31" s="37" t="s">
         <v>28</v>
       </c>
       <c r="G31" s="34" t="s">
+        <v>148</v>
+      </c>
+      <c r="H31" s="34" t="s">
         <v>149</v>
       </c>
-      <c r="H31" s="34" t="s">
+      <c r="I31" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J31" s="34" t="s">
         <v>150</v>
-      </c>
-      <c r="I31" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J31" s="34" t="s">
-        <v>151</v>
       </c>
       <c r="K31" s="34" t="s">
         <v>31</v>
@@ -3505,28 +3508,28 @@
         <v>23</v>
       </c>
       <c r="C32" s="36" t="s">
+        <v>151</v>
+      </c>
+      <c r="D32" s="37" t="s">
         <v>152</v>
       </c>
-      <c r="D32" s="37" t="s">
+      <c r="E32" s="37" t="s">
         <v>153</v>
-      </c>
-      <c r="E32" s="37" t="s">
-        <v>154</v>
       </c>
       <c r="F32" s="37" t="s">
         <v>28</v>
       </c>
       <c r="G32" s="37" t="s">
+        <v>154</v>
+      </c>
+      <c r="H32" s="37" t="s">
         <v>155</v>
       </c>
-      <c r="H32" s="37" t="s">
+      <c r="I32" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J32" s="37" t="s">
         <v>156</v>
-      </c>
-      <c r="I32" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J32" s="37" t="s">
-        <v>157</v>
       </c>
       <c r="K32" s="37" t="s">
         <v>31</v>
@@ -3561,28 +3564,28 @@
         <v>24</v>
       </c>
       <c r="C33" s="33" t="s">
+        <v>157</v>
+      </c>
+      <c r="D33" s="34" t="s">
         <v>158</v>
       </c>
-      <c r="D33" s="34" t="s">
+      <c r="E33" s="34" t="s">
         <v>159</v>
       </c>
-      <c r="E33" s="34" t="s">
+      <c r="F33" s="34" t="s">
         <v>160</v>
       </c>
-      <c r="F33" s="34" t="s">
+      <c r="G33" s="34" t="s">
         <v>161</v>
       </c>
-      <c r="G33" s="34" t="s">
+      <c r="H33" s="34" t="s">
         <v>162</v>
       </c>
-      <c r="H33" s="34" t="s">
+      <c r="I33" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J33" s="34" t="s">
         <v>163</v>
-      </c>
-      <c r="I33" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J33" s="34" t="s">
-        <v>164</v>
       </c>
       <c r="K33" s="34" t="s">
         <v>31</v>
@@ -3617,28 +3620,28 @@
         <v>25</v>
       </c>
       <c r="C34" s="36" t="s">
+        <v>164</v>
+      </c>
+      <c r="D34" s="37" t="s">
         <v>165</v>
       </c>
-      <c r="D34" s="37" t="s">
+      <c r="E34" s="37" t="s">
         <v>166</v>
       </c>
-      <c r="E34" s="37" t="s">
+      <c r="F34" s="37" t="s">
         <v>167</v>
       </c>
-      <c r="F34" s="37" t="s">
+      <c r="G34" s="37" t="s">
         <v>168</v>
       </c>
-      <c r="G34" s="37" t="s">
+      <c r="H34" s="37" t="s">
         <v>169</v>
       </c>
-      <c r="H34" s="37" t="s">
+      <c r="I34" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="J34" s="37" t="s">
         <v>170</v>
-      </c>
-      <c r="I34" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="J34" s="37" t="s">
-        <v>171</v>
       </c>
       <c r="K34" s="37" t="s">
         <v>31</v>
@@ -3673,28 +3676,28 @@
         <v>26</v>
       </c>
       <c r="C35" s="33" t="s">
+        <v>171</v>
+      </c>
+      <c r="D35" s="34" t="s">
         <v>172</v>
       </c>
-      <c r="D35" s="34" t="s">
+      <c r="E35" s="34" t="s">
         <v>173</v>
       </c>
-      <c r="E35" s="34" t="s">
+      <c r="F35" s="34" t="s">
         <v>174</v>
       </c>
-      <c r="F35" s="34" t="s">
+      <c r="G35" s="34" t="s">
         <v>175</v>
       </c>
-      <c r="G35" s="34" t="s">
+      <c r="H35" s="34" t="s">
         <v>176</v>
       </c>
-      <c r="H35" s="34" t="s">
+      <c r="I35" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J35" s="34" t="s">
         <v>177</v>
-      </c>
-      <c r="I35" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J35" s="34" t="s">
-        <v>178</v>
       </c>
       <c r="K35" s="34" t="s">
         <v>31</v>
@@ -3729,31 +3732,31 @@
         <v>27</v>
       </c>
       <c r="C36" s="33" t="s">
+        <v>178</v>
+      </c>
+      <c r="D36" s="37" t="s">
         <v>179</v>
       </c>
-      <c r="D36" s="37" t="s">
+      <c r="E36" s="37" t="s">
         <v>180</v>
       </c>
-      <c r="E36" s="37" t="s">
+      <c r="F36" s="37" t="s">
         <v>181</v>
       </c>
-      <c r="F36" s="37" t="s">
+      <c r="G36" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G36" s="37" t="s">
+      <c r="H36" s="37" t="s">
         <v>183</v>
       </c>
-      <c r="H36" s="37" t="s">
+      <c r="I36" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="J36" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I36" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="J36" s="37" t="s">
+      <c r="K36" s="37" t="s">
         <v>185</v>
-      </c>
-      <c r="K36" s="37" t="s">
-        <v>186</v>
       </c>
       <c r="L36" s="37">
         <v>4</v>
@@ -3785,31 +3788,31 @@
         <v>28</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D37" s="34" t="s">
+        <v>186</v>
+      </c>
+      <c r="E37" s="34" t="s">
         <v>187</v>
-      </c>
-      <c r="E37" s="34" t="s">
-        <v>188</v>
       </c>
       <c r="F37" s="34" t="s">
         <v>28</v>
       </c>
       <c r="G37" s="34" t="s">
+        <v>188</v>
+      </c>
+      <c r="H37" s="34" t="s">
         <v>189</v>
       </c>
-      <c r="H37" s="34" t="s">
+      <c r="I37" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J37" s="34" t="s">
         <v>190</v>
       </c>
-      <c r="I37" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J37" s="34" t="s">
+      <c r="K37" s="34" t="s">
         <v>191</v>
-      </c>
-      <c r="K37" s="34" t="s">
-        <v>192</v>
       </c>
       <c r="L37" s="34">
         <v>2</v>
@@ -3841,19 +3844,19 @@
         <v>29</v>
       </c>
       <c r="C38" s="33" t="s">
+        <v>192</v>
+      </c>
+      <c r="D38" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="D38" s="37" t="s">
+      <c r="E38" s="37" t="s">
         <v>194</v>
       </c>
-      <c r="E38" s="37" t="s">
+      <c r="F38" s="37" t="s">
         <v>195</v>
       </c>
-      <c r="F38" s="37" t="s">
+      <c r="G38" s="37" t="s">
         <v>196</v>
-      </c>
-      <c r="G38" s="37" t="s">
-        <v>197</v>
       </c>
       <c r="H38" s="37" t="s">
         <v>39</v>
@@ -3862,10 +3865,10 @@
         <v>31</v>
       </c>
       <c r="J38" s="37" t="s">
+        <v>197</v>
+      </c>
+      <c r="K38" s="37" t="s">
         <v>198</v>
-      </c>
-      <c r="K38" s="37" t="s">
-        <v>199</v>
       </c>
       <c r="L38" s="37">
         <v>3</v>
@@ -3897,19 +3900,19 @@
         <v>30</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D39" s="34" t="s">
+        <v>199</v>
+      </c>
+      <c r="E39" s="34" t="s">
         <v>200</v>
       </c>
-      <c r="E39" s="34" t="s">
+      <c r="F39" s="34" t="s">
+        <v>195</v>
+      </c>
+      <c r="G39" s="34" t="s">
         <v>201</v>
-      </c>
-      <c r="F39" s="34" t="s">
-        <v>196</v>
-      </c>
-      <c r="G39" s="34" t="s">
-        <v>202</v>
       </c>
       <c r="H39" s="34" t="s">
         <v>39</v>
@@ -3918,10 +3921,10 @@
         <v>31</v>
       </c>
       <c r="J39" s="34" t="s">
+        <v>202</v>
+      </c>
+      <c r="K39" s="34" t="s">
         <v>203</v>
-      </c>
-      <c r="K39" s="34" t="s">
-        <v>204</v>
       </c>
       <c r="L39" s="34">
         <v>6</v>
@@ -3953,19 +3956,19 @@
         <v>31</v>
       </c>
       <c r="C40" s="36" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D40" s="37" t="s">
+        <v>204</v>
+      </c>
+      <c r="E40" s="37" t="s">
         <v>205</v>
       </c>
-      <c r="E40" s="37" t="s">
+      <c r="F40" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="G40" s="37" t="s">
         <v>206</v>
-      </c>
-      <c r="F40" s="37" t="s">
-        <v>196</v>
-      </c>
-      <c r="G40" s="37" t="s">
-        <v>207</v>
       </c>
       <c r="H40" s="37" t="s">
         <v>39</v>
@@ -3974,10 +3977,10 @@
         <v>31</v>
       </c>
       <c r="J40" s="37" t="s">
+        <v>207</v>
+      </c>
+      <c r="K40" s="37" t="s">
         <v>208</v>
-      </c>
-      <c r="K40" s="37" t="s">
-        <v>209</v>
       </c>
       <c r="L40" s="37">
         <v>4</v>
@@ -4009,19 +4012,19 @@
         <v>32</v>
       </c>
       <c r="C41" s="36" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D41" s="34" t="s">
+        <v>209</v>
+      </c>
+      <c r="E41" s="34" t="s">
         <v>210</v>
       </c>
-      <c r="E41" s="34" t="s">
+      <c r="F41" s="34" t="s">
+        <v>195</v>
+      </c>
+      <c r="G41" s="34" t="s">
         <v>211</v>
-      </c>
-      <c r="F41" s="34" t="s">
-        <v>196</v>
-      </c>
-      <c r="G41" s="34" t="s">
-        <v>212</v>
       </c>
       <c r="H41" s="34" t="s">
         <v>39</v>
@@ -4030,10 +4033,10 @@
         <v>31</v>
       </c>
       <c r="J41" s="34" t="s">
+        <v>212</v>
+      </c>
+      <c r="K41" s="34" t="s">
         <v>213</v>
-      </c>
-      <c r="K41" s="34" t="s">
-        <v>214</v>
       </c>
       <c r="L41" s="34">
         <v>2</v>
@@ -4065,19 +4068,19 @@
         <v>33</v>
       </c>
       <c r="C42" s="36" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D42" s="37" t="s">
+        <v>214</v>
+      </c>
+      <c r="E42" s="37" t="s">
         <v>215</v>
       </c>
-      <c r="E42" s="37" t="s">
+      <c r="F42" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="G42" s="37" t="s">
         <v>216</v>
-      </c>
-      <c r="F42" s="37" t="s">
-        <v>196</v>
-      </c>
-      <c r="G42" s="37" t="s">
-        <v>217</v>
       </c>
       <c r="H42" s="37" t="s">
         <v>39</v>
@@ -4086,10 +4089,10 @@
         <v>31</v>
       </c>
       <c r="J42" s="37" t="s">
+        <v>217</v>
+      </c>
+      <c r="K42" s="37" t="s">
         <v>218</v>
-      </c>
-      <c r="K42" s="37" t="s">
-        <v>219</v>
       </c>
       <c r="L42" s="37">
         <v>3</v>
@@ -4121,31 +4124,31 @@
         <v>34</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D43" s="34" t="s">
+        <v>219</v>
+      </c>
+      <c r="E43" s="34" t="s">
         <v>220</v>
       </c>
-      <c r="E43" s="34" t="s">
+      <c r="F43" s="34" t="s">
+        <v>195</v>
+      </c>
+      <c r="G43" s="34" t="s">
         <v>221</v>
       </c>
-      <c r="F43" s="34" t="s">
-        <v>196</v>
-      </c>
-      <c r="G43" s="34" t="s">
+      <c r="H43" s="34" t="s">
         <v>222</v>
       </c>
-      <c r="H43" s="34" t="s">
+      <c r="I43" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="J43" s="34" t="s">
         <v>223</v>
       </c>
-      <c r="I43" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="J43" s="34" t="s">
+      <c r="K43" s="34" t="s">
         <v>224</v>
-      </c>
-      <c r="K43" s="34" t="s">
-        <v>225</v>
       </c>
       <c r="L43" s="34">
         <v>6</v>
@@ -4177,19 +4180,19 @@
         <v>35</v>
       </c>
       <c r="C44" s="36" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D44" s="37" t="s">
+        <v>225</v>
+      </c>
+      <c r="E44" s="37" t="s">
         <v>226</v>
       </c>
-      <c r="E44" s="37" t="s">
+      <c r="F44" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="G44" s="37" t="s">
         <v>227</v>
-      </c>
-      <c r="F44" s="37" t="s">
-        <v>196</v>
-      </c>
-      <c r="G44" s="37" t="s">
-        <v>228</v>
       </c>
       <c r="H44" s="37" t="s">
         <v>39</v>
@@ -4198,10 +4201,10 @@
         <v>31</v>
       </c>
       <c r="J44" s="37" t="s">
+        <v>228</v>
+      </c>
+      <c r="K44" s="37" t="s">
         <v>229</v>
-      </c>
-      <c r="K44" s="37" t="s">
-        <v>230</v>
       </c>
       <c r="L44" s="37">
         <v>2</v>
@@ -4233,19 +4236,19 @@
         <v>36</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D45" s="34" t="s">
+        <v>230</v>
+      </c>
+      <c r="E45" s="34" t="s">
         <v>231</v>
       </c>
-      <c r="E45" s="34" t="s">
+      <c r="F45" s="34" t="s">
+        <v>195</v>
+      </c>
+      <c r="G45" s="34" t="s">
         <v>232</v>
-      </c>
-      <c r="F45" s="34" t="s">
-        <v>196</v>
-      </c>
-      <c r="G45" s="34" t="s">
-        <v>233</v>
       </c>
       <c r="H45" s="34" t="s">
         <v>39</v>
@@ -4254,10 +4257,10 @@
         <v>31</v>
       </c>
       <c r="J45" s="34" t="s">
+        <v>233</v>
+      </c>
+      <c r="K45" s="34" t="s">
         <v>234</v>
-      </c>
-      <c r="K45" s="34" t="s">
-        <v>235</v>
       </c>
       <c r="L45" s="34">
         <v>3</v>
@@ -4289,19 +4292,19 @@
         <v>37</v>
       </c>
       <c r="C46" s="36" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D46" s="37" t="s">
+        <v>235</v>
+      </c>
+      <c r="E46" s="37" t="s">
         <v>236</v>
       </c>
-      <c r="E46" s="37" t="s">
+      <c r="F46" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="G46" s="37" t="s">
         <v>237</v>
-      </c>
-      <c r="F46" s="37" t="s">
-        <v>196</v>
-      </c>
-      <c r="G46" s="37" t="s">
-        <v>238</v>
       </c>
       <c r="H46" s="37" t="s">
         <v>39</v>
@@ -4310,10 +4313,10 @@
         <v>31</v>
       </c>
       <c r="J46" s="37" t="s">
+        <v>238</v>
+      </c>
+      <c r="K46" s="37" t="s">
         <v>239</v>
-      </c>
-      <c r="K46" s="37" t="s">
-        <v>240</v>
       </c>
       <c r="L46" s="37">
         <v>1</v>
@@ -4345,19 +4348,19 @@
         <v>38</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D47" s="34" t="s">
+        <v>240</v>
+      </c>
+      <c r="E47" s="34" t="s">
         <v>241</v>
       </c>
-      <c r="E47" s="34" t="s">
+      <c r="F47" s="34" t="s">
+        <v>195</v>
+      </c>
+      <c r="G47" s="34" t="s">
         <v>242</v>
-      </c>
-      <c r="F47" s="34" t="s">
-        <v>196</v>
-      </c>
-      <c r="G47" s="34" t="s">
-        <v>243</v>
       </c>
       <c r="H47" s="34" t="s">
         <v>39</v>
@@ -4366,10 +4369,10 @@
         <v>31</v>
       </c>
       <c r="J47" s="34" t="s">
+        <v>243</v>
+      </c>
+      <c r="K47" s="34" t="s">
         <v>244</v>
-      </c>
-      <c r="K47" s="34" t="s">
-        <v>245</v>
       </c>
       <c r="L47" s="34">
         <v>1</v>
@@ -4382,7 +4385,7 @@
         <v>100</v>
       </c>
       <c r="O47" s="51" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="P47" s="52">
         <v>1.1999999999999999E-3</v>
@@ -4401,31 +4404,31 @@
         <v>39</v>
       </c>
       <c r="C48" s="36" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D48" s="37" t="s">
+        <v>246</v>
+      </c>
+      <c r="E48" s="37" t="s">
         <v>247</v>
       </c>
-      <c r="E48" s="37" t="s">
+      <c r="F48" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="G48" s="38" t="s">
         <v>248</v>
-      </c>
-      <c r="F48" s="37" t="s">
-        <v>196</v>
-      </c>
-      <c r="G48" s="38" t="s">
-        <v>249</v>
       </c>
       <c r="H48" s="37" t="s">
         <v>39</v>
       </c>
       <c r="I48" s="37" t="s">
+        <v>249</v>
+      </c>
+      <c r="J48" s="37" t="s">
         <v>250</v>
       </c>
-      <c r="J48" s="37" t="s">
+      <c r="K48" s="37" t="s">
         <v>251</v>
-      </c>
-      <c r="K48" s="37" t="s">
-        <v>252</v>
       </c>
       <c r="L48" s="37">
         <v>6</v>
@@ -4457,31 +4460,31 @@
         <v>40</v>
       </c>
       <c r="C49" s="33" t="s">
+        <v>252</v>
+      </c>
+      <c r="D49" s="34" t="s">
         <v>253</v>
       </c>
-      <c r="D49" s="34" t="s">
+      <c r="E49" s="34" t="s">
         <v>254</v>
-      </c>
-      <c r="E49" s="34" t="s">
-        <v>255</v>
       </c>
       <c r="F49" s="34" t="s">
         <v>28</v>
       </c>
       <c r="G49" s="34" t="s">
+        <v>255</v>
+      </c>
+      <c r="H49" s="34" t="s">
         <v>256</v>
       </c>
-      <c r="H49" s="34" t="s">
+      <c r="I49" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J49" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="I49" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J49" s="34" t="s">
-        <v>258</v>
-      </c>
       <c r="K49" s="34" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="L49" s="34">
         <v>2</v>
@@ -4513,28 +4516,28 @@
         <v>41</v>
       </c>
       <c r="C50" s="36" t="s">
+        <v>258</v>
+      </c>
+      <c r="D50" s="37" t="s">
         <v>259</v>
       </c>
-      <c r="D50" s="37" t="s">
+      <c r="E50" s="37" t="s">
         <v>260</v>
-      </c>
-      <c r="E50" s="37" t="s">
-        <v>261</v>
       </c>
       <c r="F50" s="34" t="s">
         <v>28</v>
       </c>
       <c r="G50" s="37" t="s">
+        <v>261</v>
+      </c>
+      <c r="H50" s="37" t="s">
         <v>262</v>
       </c>
-      <c r="H50" s="37" t="s">
+      <c r="I50" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J50" s="37" t="s">
         <v>263</v>
-      </c>
-      <c r="I50" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J50" s="37" t="s">
-        <v>264</v>
       </c>
       <c r="K50" s="37" t="s">
         <v>31</v>
@@ -4569,28 +4572,28 @@
         <v>42</v>
       </c>
       <c r="C51" s="33" t="s">
+        <v>264</v>
+      </c>
+      <c r="D51" s="34" t="s">
         <v>265</v>
       </c>
-      <c r="D51" s="34" t="s">
+      <c r="E51" s="34" t="s">
         <v>266</v>
-      </c>
-      <c r="E51" s="34" t="s">
-        <v>267</v>
       </c>
       <c r="F51" s="34" t="s">
         <v>28</v>
       </c>
       <c r="G51" s="34" t="s">
+        <v>267</v>
+      </c>
+      <c r="H51" s="34" t="s">
         <v>268</v>
       </c>
-      <c r="H51" s="34" t="s">
+      <c r="I51" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J51" s="34" t="s">
         <v>269</v>
-      </c>
-      <c r="I51" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J51" s="34" t="s">
-        <v>270</v>
       </c>
       <c r="K51" s="34" t="s">
         <v>31</v>
@@ -4625,28 +4628,28 @@
         <v>43</v>
       </c>
       <c r="C52" s="36" t="s">
+        <v>270</v>
+      </c>
+      <c r="D52" s="37" t="s">
         <v>271</v>
       </c>
-      <c r="D52" s="37" t="s">
+      <c r="E52" s="37" t="s">
         <v>272</v>
-      </c>
-      <c r="E52" s="37" t="s">
-        <v>273</v>
       </c>
       <c r="F52" s="34" t="s">
         <v>28</v>
       </c>
       <c r="G52" s="37" t="s">
+        <v>273</v>
+      </c>
+      <c r="H52" s="37" t="s">
         <v>274</v>
       </c>
-      <c r="H52" s="37" t="s">
+      <c r="I52" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="J52" s="37" t="s">
         <v>275</v>
-      </c>
-      <c r="I52" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="J52" s="37" t="s">
-        <v>276</v>
       </c>
       <c r="K52" s="37" t="s">
         <v>31</v>
@@ -4681,22 +4684,22 @@
         <v>44</v>
       </c>
       <c r="C53" s="33" t="s">
+        <v>276</v>
+      </c>
+      <c r="D53" s="34" t="s">
         <v>277</v>
       </c>
-      <c r="D53" s="34" t="s">
+      <c r="E53" s="34" t="s">
         <v>278</v>
-      </c>
-      <c r="E53" s="34" t="s">
-        <v>279</v>
       </c>
       <c r="F53" s="34" t="s">
         <v>28</v>
       </c>
       <c r="G53" s="34" t="s">
+        <v>279</v>
+      </c>
+      <c r="H53" s="34" t="s">
         <v>280</v>
-      </c>
-      <c r="H53" s="34" t="s">
-        <v>281</v>
       </c>
       <c r="I53" s="34" t="s">
         <v>31</v>
@@ -4718,7 +4721,7 @@
         <v>6</v>
       </c>
       <c r="O53" s="51" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="P53" s="52">
         <v>2.76</v>
@@ -4737,28 +4740,28 @@
         <v>45</v>
       </c>
       <c r="C54" s="36" t="s">
+        <v>282</v>
+      </c>
+      <c r="D54" s="37" t="s">
         <v>283</v>
       </c>
-      <c r="D54" s="37" t="s">
+      <c r="E54" s="37" t="s">
         <v>284</v>
       </c>
-      <c r="E54" s="37" t="s">
+      <c r="F54" s="37" t="s">
         <v>285</v>
       </c>
-      <c r="F54" s="37" t="s">
+      <c r="G54" s="37" t="s">
         <v>286</v>
       </c>
-      <c r="G54" s="37" t="s">
+      <c r="H54" s="37" t="s">
         <v>287</v>
       </c>
-      <c r="H54" s="37" t="s">
+      <c r="I54" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="J54" s="37" t="s">
         <v>288</v>
-      </c>
-      <c r="I54" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="J54" s="37" t="s">
-        <v>289</v>
       </c>
       <c r="K54" s="37" t="s">
         <v>31</v>
@@ -4793,28 +4796,28 @@
         <v>46</v>
       </c>
       <c r="C55" s="33" t="s">
+        <v>289</v>
+      </c>
+      <c r="D55" s="34" t="s">
         <v>290</v>
       </c>
-      <c r="D55" s="34" t="s">
+      <c r="E55" s="34" t="s">
+        <v>284</v>
+      </c>
+      <c r="F55" s="34" t="s">
+        <v>285</v>
+      </c>
+      <c r="G55" s="34" t="s">
         <v>291</v>
       </c>
-      <c r="E55" s="34" t="s">
-        <v>285</v>
-      </c>
-      <c r="F55" s="34" t="s">
-        <v>286</v>
-      </c>
-      <c r="G55" s="34" t="s">
+      <c r="H55" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="I55" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J55" s="34" t="s">
         <v>292</v>
-      </c>
-      <c r="H55" s="37" t="s">
-        <v>288</v>
-      </c>
-      <c r="I55" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J55" s="34" t="s">
-        <v>293</v>
       </c>
       <c r="K55" s="34" t="s">
         <v>31</v>
@@ -4849,28 +4852,28 @@
         <v>47</v>
       </c>
       <c r="C56" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="D56" s="37" t="s">
         <v>294</v>
       </c>
-      <c r="D56" s="37" t="s">
+      <c r="E56" s="37" t="s">
         <v>295</v>
       </c>
-      <c r="E56" s="37" t="s">
+      <c r="F56" s="37" t="s">
         <v>296</v>
       </c>
-      <c r="F56" s="37" t="s">
+      <c r="G56" s="37" t="s">
         <v>297</v>
       </c>
-      <c r="G56" s="37" t="s">
+      <c r="H56" s="37" t="s">
         <v>298</v>
       </c>
-      <c r="H56" s="37" t="s">
+      <c r="I56" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J56" s="37" t="s">
         <v>299</v>
-      </c>
-      <c r="I56" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J56" s="37" t="s">
-        <v>300</v>
       </c>
       <c r="K56" s="34" t="s">
         <v>31</v>
@@ -4905,28 +4908,28 @@
         <v>48</v>
       </c>
       <c r="C57" s="33" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D57" s="34" t="s">
+        <v>300</v>
+      </c>
+      <c r="E57" s="34" t="s">
         <v>301</v>
       </c>
-      <c r="E57" s="34" t="s">
+      <c r="F57" s="34" t="s">
         <v>302</v>
       </c>
-      <c r="F57" s="34" t="s">
+      <c r="G57" s="34" t="s">
         <v>303</v>
       </c>
-      <c r="G57" s="34" t="s">
+      <c r="H57" s="37" t="s">
         <v>304</v>
       </c>
-      <c r="H57" s="37" t="s">
+      <c r="I57" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J57" s="34" t="s">
         <v>305</v>
-      </c>
-      <c r="I57" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J57" s="34" t="s">
-        <v>306</v>
       </c>
       <c r="K57" s="34" t="s">
         <v>31</v>
@@ -4961,28 +4964,28 @@
         <v>49</v>
       </c>
       <c r="C58" s="36" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D58" s="37" t="s">
+        <v>306</v>
+      </c>
+      <c r="E58" s="37" t="s">
         <v>307</v>
       </c>
-      <c r="E58" s="37" t="s">
+      <c r="F58" s="37" t="s">
         <v>308</v>
       </c>
-      <c r="F58" s="37" t="s">
+      <c r="G58" s="37" t="s">
         <v>309</v>
       </c>
-      <c r="G58" s="37" t="s">
+      <c r="H58" s="37" t="s">
         <v>310</v>
       </c>
-      <c r="H58" s="37" t="s">
+      <c r="I58" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J58" s="37" t="s">
         <v>311</v>
-      </c>
-      <c r="I58" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J58" s="37" t="s">
-        <v>312</v>
       </c>
       <c r="K58" s="34" t="s">
         <v>31</v>
@@ -5017,28 +5020,28 @@
         <v>50</v>
       </c>
       <c r="C59" s="33" t="s">
+        <v>312</v>
+      </c>
+      <c r="D59" s="34" t="s">
         <v>313</v>
       </c>
-      <c r="D59" s="34" t="s">
+      <c r="E59" s="34" t="s">
         <v>314</v>
       </c>
-      <c r="E59" s="34" t="s">
+      <c r="F59" s="34" t="s">
+        <v>167</v>
+      </c>
+      <c r="G59" s="34" t="s">
         <v>315</v>
       </c>
-      <c r="F59" s="34" t="s">
-        <v>168</v>
-      </c>
-      <c r="G59" s="34" t="s">
+      <c r="H59" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="I59" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J59" s="34" t="s">
         <v>316</v>
-      </c>
-      <c r="H59" s="34" t="s">
-        <v>170</v>
-      </c>
-      <c r="I59" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J59" s="34" t="s">
-        <v>317</v>
       </c>
       <c r="K59" s="34" t="s">
         <v>31</v>
@@ -5073,28 +5076,28 @@
         <v>51</v>
       </c>
       <c r="C60" s="33" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D60" s="34" t="s">
         <v>31</v>
       </c>
       <c r="E60" s="34" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="F60" s="34" t="s">
         <v>28</v>
       </c>
       <c r="G60" s="34" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H60" s="34" t="s">
+        <v>322</v>
+      </c>
+      <c r="I60" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J60" s="34" t="s">
         <v>323</v>
-      </c>
-      <c r="I60" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J60" s="34" t="s">
-        <v>324</v>
       </c>
       <c r="K60" s="34" t="s">
         <v>31</v>
@@ -5129,28 +5132,28 @@
         <v>52</v>
       </c>
       <c r="C61" s="33" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D61" s="34" t="s">
         <v>31</v>
       </c>
       <c r="E61" s="34" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F61" s="34" t="s">
         <v>28</v>
       </c>
       <c r="G61" s="34" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="H61" s="34" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="I61" s="34" t="s">
         <v>31</v>
       </c>
       <c r="J61" s="34" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="K61" s="34" t="s">
         <v>31</v>
@@ -5185,28 +5188,28 @@
         <v>53</v>
       </c>
       <c r="C62" s="33" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D62" s="34" t="s">
         <v>31</v>
       </c>
       <c r="E62" s="34" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F62" s="34" t="s">
         <v>28</v>
       </c>
       <c r="G62" s="34" t="s">
+        <v>327</v>
+      </c>
+      <c r="H62" s="34" t="s">
         <v>328</v>
       </c>
-      <c r="H62" s="34" t="s">
+      <c r="I62" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="J62" s="34" t="s">
         <v>329</v>
-      </c>
-      <c r="I62" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="J62" s="34" t="s">
-        <v>330</v>
       </c>
       <c r="K62" s="34" t="s">
         <v>31</v>
@@ -5241,19 +5244,19 @@
         <v>54</v>
       </c>
       <c r="C63" s="33" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D63" s="34" t="s">
         <v>31</v>
       </c>
       <c r="E63" s="34" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F63" s="34" t="s">
         <v>31</v>
       </c>
       <c r="G63" s="34" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="H63" s="34" t="s">
         <v>31</v>
@@ -5278,7 +5281,7 @@
         <v>5</v>
       </c>
       <c r="O63" s="51" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="P63" s="52">
         <v>2</v>
@@ -5305,13 +5308,13 @@
       <c r="L64" s="46"/>
       <c r="M64" s="46"/>
       <c r="N64" s="66" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="O64" s="67"/>
       <c r="P64" s="67"/>
       <c r="Q64" s="59">
         <f>SUM(Q10:Q63)</f>
-        <v>131.56720000000001</v>
+        <v>128.11520000000002</v>
       </c>
       <c r="R64" s="70"/>
       <c r="S64" s="71"/>
@@ -5331,13 +5334,13 @@
       <c r="L65" s="50"/>
       <c r="M65" s="50"/>
       <c r="N65" s="66" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="O65" s="67"/>
       <c r="P65" s="67"/>
       <c r="Q65" s="60">
         <f>Q64/5</f>
-        <v>26.313440000000003</v>
+        <v>25.623040000000003</v>
       </c>
       <c r="R65" s="72"/>
       <c r="S65" s="73"/>
@@ -5366,43 +5369,43 @@
     <hyperlink ref="O24" r:id="rId13"/>
     <hyperlink ref="O25" r:id="rId14"/>
     <hyperlink ref="O26" r:id="rId15"/>
-    <hyperlink ref="O28" r:id="rId16"/>
-    <hyperlink ref="O30" r:id="rId17"/>
-    <hyperlink ref="O31" r:id="rId18"/>
-    <hyperlink ref="O32" r:id="rId19"/>
-    <hyperlink ref="O33" r:id="rId20"/>
-    <hyperlink ref="O35" r:id="rId21"/>
-    <hyperlink ref="O36" r:id="rId22"/>
-    <hyperlink ref="O37" r:id="rId23"/>
-    <hyperlink ref="O38" r:id="rId24"/>
-    <hyperlink ref="O39" r:id="rId25"/>
-    <hyperlink ref="O40" r:id="rId26"/>
-    <hyperlink ref="O41" r:id="rId27"/>
-    <hyperlink ref="O42" r:id="rId28"/>
-    <hyperlink ref="O43" r:id="rId29"/>
-    <hyperlink ref="O44" r:id="rId30"/>
-    <hyperlink ref="O45" r:id="rId31"/>
-    <hyperlink ref="O46" r:id="rId32"/>
-    <hyperlink ref="O47" r:id="rId33"/>
-    <hyperlink ref="O49" r:id="rId34"/>
-    <hyperlink ref="O50" r:id="rId35"/>
-    <hyperlink ref="O51" r:id="rId36"/>
-    <hyperlink ref="O52" r:id="rId37"/>
-    <hyperlink ref="O54" r:id="rId38"/>
-    <hyperlink ref="O56" r:id="rId39"/>
-    <hyperlink ref="O58" r:id="rId40"/>
-    <hyperlink ref="O59" r:id="rId41"/>
-    <hyperlink ref="O13" r:id="rId42"/>
-    <hyperlink ref="O34" r:id="rId43"/>
-    <hyperlink ref="O48" r:id="rId44"/>
-    <hyperlink ref="O53" r:id="rId45"/>
-    <hyperlink ref="O55" r:id="rId46"/>
-    <hyperlink ref="O19" r:id="rId47"/>
-    <hyperlink ref="O57" r:id="rId48"/>
-    <hyperlink ref="O60" r:id="rId49"/>
-    <hyperlink ref="O61" r:id="rId50"/>
-    <hyperlink ref="O62" r:id="rId51"/>
-    <hyperlink ref="O63" r:id="rId52"/>
+    <hyperlink ref="O30" r:id="rId16"/>
+    <hyperlink ref="O31" r:id="rId17"/>
+    <hyperlink ref="O32" r:id="rId18"/>
+    <hyperlink ref="O33" r:id="rId19"/>
+    <hyperlink ref="O35" r:id="rId20"/>
+    <hyperlink ref="O36" r:id="rId21"/>
+    <hyperlink ref="O37" r:id="rId22"/>
+    <hyperlink ref="O38" r:id="rId23"/>
+    <hyperlink ref="O39" r:id="rId24"/>
+    <hyperlink ref="O40" r:id="rId25"/>
+    <hyperlink ref="O41" r:id="rId26"/>
+    <hyperlink ref="O42" r:id="rId27"/>
+    <hyperlink ref="O43" r:id="rId28"/>
+    <hyperlink ref="O44" r:id="rId29"/>
+    <hyperlink ref="O45" r:id="rId30"/>
+    <hyperlink ref="O46" r:id="rId31"/>
+    <hyperlink ref="O47" r:id="rId32"/>
+    <hyperlink ref="O49" r:id="rId33"/>
+    <hyperlink ref="O50" r:id="rId34"/>
+    <hyperlink ref="O51" r:id="rId35"/>
+    <hyperlink ref="O52" r:id="rId36"/>
+    <hyperlink ref="O54" r:id="rId37"/>
+    <hyperlink ref="O56" r:id="rId38"/>
+    <hyperlink ref="O58" r:id="rId39"/>
+    <hyperlink ref="O59" r:id="rId40"/>
+    <hyperlink ref="O13" r:id="rId41"/>
+    <hyperlink ref="O34" r:id="rId42"/>
+    <hyperlink ref="O48" r:id="rId43"/>
+    <hyperlink ref="O53" r:id="rId44"/>
+    <hyperlink ref="O55" r:id="rId45"/>
+    <hyperlink ref="O19" r:id="rId46"/>
+    <hyperlink ref="O57" r:id="rId47"/>
+    <hyperlink ref="O60" r:id="rId48"/>
+    <hyperlink ref="O61" r:id="rId49"/>
+    <hyperlink ref="O62" r:id="rId50"/>
+    <hyperlink ref="O63" r:id="rId51"/>
+    <hyperlink ref="O28" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>